<commit_message>
style: perfect typography, column sizing and symmetric KPI layouts across Excel, Google Sheet and Web
</commit_message>
<xml_diff>
--- a/docs/RevOps_Platform_Demo_Sample.xlsx
+++ b/docs/RevOps_Platform_Demo_Sample.xlsx
@@ -304,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -448,6 +448,9 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -519,6 +522,9 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -547,6 +553,12 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1632,7 +1644,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="58" customHeight="1">
       <c r="A9" s="26" t="n">
         <v>1</v>
       </c>
@@ -1670,7 +1682,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
+    <row r="10" ht="58" customHeight="1">
       <c r="A10" s="26" t="n">
         <v>2</v>
       </c>
@@ -1708,7 +1720,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="58" customHeight="1">
       <c r="A11" s="26" t="n">
         <v>3</v>
       </c>
@@ -1746,7 +1758,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1">
+    <row r="12" ht="58" customHeight="1">
       <c r="A12" s="26" t="n">
         <v>4</v>
       </c>
@@ -1784,7 +1796,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="58" customHeight="1">
       <c r="A13" s="26" t="n">
         <v>5</v>
       </c>
@@ -1967,14 +1979,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
@@ -2189,48 +2201,48 @@
       <c r="U6" s="58" t="n"/>
       <c r="V6" s="58" t="n"/>
     </row>
-    <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="25" t="inlineStr">
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="59" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="59" t="inlineStr">
         <is>
           <t>Менеджер ОП</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
+      <c r="C7" s="59" t="inlineStr">
         <is>
           <t>Звонков</t>
         </is>
       </c>
-      <c r="D7" s="25" t="inlineStr">
+      <c r="D7" s="59" t="inlineStr">
         <is>
           <t>Ср. балл /13</t>
         </is>
       </c>
-      <c r="E7" s="25" t="inlineStr">
+      <c r="E7" s="59" t="inlineStr">
         <is>
           <t>Next Step %</t>
         </is>
       </c>
-      <c r="F7" s="25" t="inlineStr">
+      <c r="F7" s="59" t="inlineStr">
         <is>
           <t>Talk/Listen (норма ≥45%)</t>
         </is>
       </c>
-      <c r="G7" s="25" t="inlineStr">
+      <c r="G7" s="59" t="inlineStr">
         <is>
           <t>Зависших сделок</t>
         </is>
       </c>
-      <c r="H7" s="25" t="inlineStr">
+      <c r="H7" s="59" t="inlineStr">
         <is>
           <t>Сумма риска (₽)</t>
         </is>
       </c>
-      <c r="I7" s="25" t="inlineStr">
+      <c r="I7" s="59" t="inlineStr">
         <is>
           <t>Грейд ИИ</t>
         </is>
@@ -2265,7 +2277,7 @@
       <c r="C8" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="59" t="n">
+      <c r="D8" s="60" t="n">
         <v>12.2</v>
       </c>
       <c r="E8" s="26" t="inlineStr">
@@ -2289,23 +2301,23 @@
           <t>⭐ А (Эталон)</t>
         </is>
       </c>
-      <c r="J8" s="60" t="inlineStr">
+      <c r="J8" s="61" t="inlineStr">
         <is>
           <t>Эталонный скрипт, рекомендован в базу знаний компании</t>
         </is>
       </c>
-      <c r="K8" s="60" t="n"/>
-      <c r="L8" s="60" t="n"/>
-      <c r="M8" s="60" t="n"/>
-      <c r="N8" s="60" t="n"/>
-      <c r="O8" s="60" t="n"/>
-      <c r="P8" s="60" t="n"/>
-      <c r="Q8" s="60" t="n"/>
-      <c r="R8" s="60" t="n"/>
-      <c r="S8" s="60" t="n"/>
-      <c r="T8" s="60" t="n"/>
-      <c r="U8" s="60" t="n"/>
-      <c r="V8" s="60" t="n"/>
+      <c r="K8" s="61" t="n"/>
+      <c r="L8" s="61" t="n"/>
+      <c r="M8" s="61" t="n"/>
+      <c r="N8" s="61" t="n"/>
+      <c r="O8" s="61" t="n"/>
+      <c r="P8" s="61" t="n"/>
+      <c r="Q8" s="61" t="n"/>
+      <c r="R8" s="61" t="n"/>
+      <c r="S8" s="61" t="n"/>
+      <c r="T8" s="61" t="n"/>
+      <c r="U8" s="61" t="n"/>
+      <c r="V8" s="61" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="26" t="n">
@@ -2319,7 +2331,7 @@
       <c r="C9" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="59" t="n">
+      <c r="D9" s="60" t="n">
         <v>10.8</v>
       </c>
       <c r="E9" s="26" t="inlineStr">
@@ -2335,7 +2347,7 @@
       <c r="G9" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="61" t="n">
+      <c r="H9" s="62" t="n">
         <v>160000</v>
       </c>
       <c r="I9" s="18" t="inlineStr">
@@ -2343,23 +2355,23 @@
           <t>🟢 B (Норма)</t>
         </is>
       </c>
-      <c r="J9" s="60" t="inlineStr">
+      <c r="J9" s="61" t="inlineStr">
         <is>
           <t>Высокая конверсия, мелкие замечания по регламенту встречи</t>
         </is>
       </c>
-      <c r="K9" s="60" t="n"/>
-      <c r="L9" s="60" t="n"/>
-      <c r="M9" s="60" t="n"/>
-      <c r="N9" s="60" t="n"/>
-      <c r="O9" s="60" t="n"/>
-      <c r="P9" s="60" t="n"/>
-      <c r="Q9" s="60" t="n"/>
-      <c r="R9" s="60" t="n"/>
-      <c r="S9" s="60" t="n"/>
-      <c r="T9" s="60" t="n"/>
-      <c r="U9" s="60" t="n"/>
-      <c r="V9" s="60" t="n"/>
+      <c r="K9" s="61" t="n"/>
+      <c r="L9" s="61" t="n"/>
+      <c r="M9" s="61" t="n"/>
+      <c r="N9" s="61" t="n"/>
+      <c r="O9" s="61" t="n"/>
+      <c r="P9" s="61" t="n"/>
+      <c r="Q9" s="61" t="n"/>
+      <c r="R9" s="61" t="n"/>
+      <c r="S9" s="61" t="n"/>
+      <c r="T9" s="61" t="n"/>
+      <c r="U9" s="61" t="n"/>
+      <c r="V9" s="61" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="26" t="n">
@@ -2373,7 +2385,7 @@
       <c r="C10" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="D10" s="62" t="n">
+      <c r="D10" s="63" t="n">
         <v>8.4</v>
       </c>
       <c r="E10" s="26" t="inlineStr">
@@ -2389,7 +2401,7 @@
       <c r="G10" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="61" t="n">
+      <c r="H10" s="62" t="n">
         <v>480000</v>
       </c>
       <c r="I10" s="20" t="inlineStr">
@@ -2397,23 +2409,23 @@
           <t>🟡 C (Зона риска)</t>
         </is>
       </c>
-      <c r="J10" s="60" t="inlineStr">
+      <c r="J10" s="61" t="inlineStr">
         <is>
           <t>Забывает фиксировать дату звонка, требуется тренинг</t>
         </is>
       </c>
-      <c r="K10" s="60" t="n"/>
-      <c r="L10" s="60" t="n"/>
-      <c r="M10" s="60" t="n"/>
-      <c r="N10" s="60" t="n"/>
-      <c r="O10" s="60" t="n"/>
-      <c r="P10" s="60" t="n"/>
-      <c r="Q10" s="60" t="n"/>
-      <c r="R10" s="60" t="n"/>
-      <c r="S10" s="60" t="n"/>
-      <c r="T10" s="60" t="n"/>
-      <c r="U10" s="60" t="n"/>
-      <c r="V10" s="60" t="n"/>
+      <c r="K10" s="61" t="n"/>
+      <c r="L10" s="61" t="n"/>
+      <c r="M10" s="61" t="n"/>
+      <c r="N10" s="61" t="n"/>
+      <c r="O10" s="61" t="n"/>
+      <c r="P10" s="61" t="n"/>
+      <c r="Q10" s="61" t="n"/>
+      <c r="R10" s="61" t="n"/>
+      <c r="S10" s="61" t="n"/>
+      <c r="T10" s="61" t="n"/>
+      <c r="U10" s="61" t="n"/>
+      <c r="V10" s="61" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="26" t="n">
@@ -2427,7 +2439,7 @@
       <c r="C11" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="D11" s="63" t="n">
+      <c r="D11" s="64" t="n">
         <v>6.2</v>
       </c>
       <c r="E11" s="26" t="inlineStr">
@@ -2443,7 +2455,7 @@
       <c r="G11" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="61" t="n">
+      <c r="H11" s="62" t="n">
         <v>1100000</v>
       </c>
       <c r="I11" s="17" t="inlineStr">
@@ -2451,23 +2463,23 @@
           <t>🔴 D (Брак речи)</t>
         </is>
       </c>
-      <c r="J11" s="60" t="inlineStr">
+      <c r="J11" s="61" t="inlineStr">
         <is>
           <t>Срыв контакта, перебивание клиента, демпинг скидок</t>
         </is>
       </c>
-      <c r="K11" s="60" t="n"/>
-      <c r="L11" s="60" t="n"/>
-      <c r="M11" s="60" t="n"/>
-      <c r="N11" s="60" t="n"/>
-      <c r="O11" s="60" t="n"/>
-      <c r="P11" s="60" t="n"/>
-      <c r="Q11" s="60" t="n"/>
-      <c r="R11" s="60" t="n"/>
-      <c r="S11" s="60" t="n"/>
-      <c r="T11" s="60" t="n"/>
-      <c r="U11" s="60" t="n"/>
-      <c r="V11" s="60" t="n"/>
+      <c r="K11" s="61" t="n"/>
+      <c r="L11" s="61" t="n"/>
+      <c r="M11" s="61" t="n"/>
+      <c r="N11" s="61" t="n"/>
+      <c r="O11" s="61" t="n"/>
+      <c r="P11" s="61" t="n"/>
+      <c r="Q11" s="61" t="n"/>
+      <c r="R11" s="61" t="n"/>
+      <c r="S11" s="61" t="n"/>
+      <c r="T11" s="61" t="n"/>
+      <c r="U11" s="61" t="n"/>
+      <c r="V11" s="61" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="26" t="n">
@@ -2481,7 +2493,7 @@
       <c r="C12" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="63" t="n">
+      <c r="D12" s="64" t="n">
         <v>5.5</v>
       </c>
       <c r="E12" s="26" t="inlineStr">
@@ -2497,7 +2509,7 @@
       <c r="G12" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="61" t="n">
+      <c r="H12" s="62" t="n">
         <v>1100000</v>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -2505,23 +2517,23 @@
           <t>🔴 D (Брак речи)</t>
         </is>
       </c>
-      <c r="J12" s="60" t="inlineStr">
+      <c r="J12" s="61" t="inlineStr">
         <is>
           <t>Режим 'автоответчика', нет попыток закрытия на встречу</t>
         </is>
       </c>
-      <c r="K12" s="60" t="n"/>
-      <c r="L12" s="60" t="n"/>
-      <c r="M12" s="60" t="n"/>
-      <c r="N12" s="60" t="n"/>
-      <c r="O12" s="60" t="n"/>
-      <c r="P12" s="60" t="n"/>
-      <c r="Q12" s="60" t="n"/>
-      <c r="R12" s="60" t="n"/>
-      <c r="S12" s="60" t="n"/>
-      <c r="T12" s="60" t="n"/>
-      <c r="U12" s="60" t="n"/>
-      <c r="V12" s="60" t="n"/>
+      <c r="K12" s="61" t="n"/>
+      <c r="L12" s="61" t="n"/>
+      <c r="M12" s="61" t="n"/>
+      <c r="N12" s="61" t="n"/>
+      <c r="O12" s="61" t="n"/>
+      <c r="P12" s="61" t="n"/>
+      <c r="Q12" s="61" t="n"/>
+      <c r="R12" s="61" t="n"/>
+      <c r="S12" s="61" t="n"/>
+      <c r="T12" s="61" t="n"/>
+      <c r="U12" s="61" t="n"/>
+      <c r="V12" s="61" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="29" t="inlineStr"/>
@@ -2530,26 +2542,26 @@
           <t>ИТОГО ПО ОТДЕЛУ ПРОДАЖ:</t>
         </is>
       </c>
-      <c r="C13" s="64">
+      <c r="C13" s="65">
         <f>SUM(C8:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="64" t="inlineStr">
+      <c r="D13" s="65" t="inlineStr">
         <is>
           <t>8.9 / 13</t>
         </is>
       </c>
-      <c r="E13" s="64" t="inlineStr">
+      <c r="E13" s="65" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
-      <c r="F13" s="64" t="inlineStr">
+      <c r="F13" s="65" t="inlineStr">
         <is>
           <t>61% / 39%</t>
         </is>
       </c>
-      <c r="G13" s="64">
+      <c r="G13" s="65">
         <f>SUM(G8:G12)</f>
         <v/>
       </c>
@@ -2557,28 +2569,28 @@
         <f>SUM(H8:H12)</f>
         <v/>
       </c>
-      <c r="I13" s="65" t="inlineStr">
+      <c r="I13" s="66" t="inlineStr">
         <is>
           <t>⚠️ РИСК</t>
         </is>
       </c>
-      <c r="J13" s="66" t="inlineStr">
+      <c r="J13" s="67" t="inlineStr">
         <is>
           <t>Требуется экспресс-коучинг по отработке возражений</t>
         </is>
       </c>
-      <c r="K13" s="66" t="n"/>
-      <c r="L13" s="66" t="n"/>
-      <c r="M13" s="66" t="n"/>
-      <c r="N13" s="66" t="n"/>
-      <c r="O13" s="66" t="n"/>
-      <c r="P13" s="66" t="n"/>
-      <c r="Q13" s="66" t="n"/>
-      <c r="R13" s="66" t="n"/>
-      <c r="S13" s="66" t="n"/>
-      <c r="T13" s="66" t="n"/>
-      <c r="U13" s="66" t="n"/>
-      <c r="V13" s="66" t="n"/>
+      <c r="K13" s="67" t="n"/>
+      <c r="L13" s="67" t="n"/>
+      <c r="M13" s="67" t="n"/>
+      <c r="N13" s="67" t="n"/>
+      <c r="O13" s="67" t="n"/>
+      <c r="P13" s="67" t="n"/>
+      <c r="Q13" s="67" t="n"/>
+      <c r="R13" s="67" t="n"/>
+      <c r="S13" s="67" t="n"/>
+      <c r="T13" s="67" t="n"/>
+      <c r="U13" s="67" t="n"/>
+      <c r="V13" s="67" t="n"/>
     </row>
     <row r="14" ht="12" customHeight="1"/>
     <row r="15" ht="24" customHeight="1">
@@ -2609,113 +2621,113 @@
       <c r="U15" s="58" t="n"/>
       <c r="V15" s="58" t="n"/>
     </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="25" t="inlineStr">
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="59" t="inlineStr">
         <is>
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B16" s="25" t="inlineStr">
+      <c r="B16" s="59" t="inlineStr">
         <is>
           <t>Сделка / Клиент</t>
         </is>
       </c>
-      <c r="C16" s="25" t="inlineStr">
+      <c r="C16" s="59" t="inlineStr">
         <is>
           <t>Менеджер</t>
         </is>
       </c>
-      <c r="D16" s="25" t="inlineStr">
+      <c r="D16" s="59" t="inlineStr">
         <is>
           <t>Сумма (₽)</t>
         </is>
       </c>
-      <c r="E16" s="25" t="inlineStr">
+      <c r="E16" s="59" t="inlineStr">
         <is>
           <t>Длит.</t>
         </is>
       </c>
-      <c r="F16" s="25" t="inlineStr">
+      <c r="F16" s="59" t="inlineStr">
         <is>
           <t>Этап CRM</t>
         </is>
       </c>
-      <c r="G16" s="25" t="inlineStr">
+      <c r="G16" s="59" t="inlineStr">
         <is>
           <t>К1 NextStep</t>
         </is>
       </c>
-      <c r="H16" s="25" t="inlineStr">
+      <c r="H16" s="59" t="inlineStr">
         <is>
           <t>К2 Иниц.</t>
         </is>
       </c>
-      <c r="I16" s="25" t="inlineStr">
+      <c r="I16" s="59" t="inlineStr">
         <is>
           <t>К3 ЛПР</t>
         </is>
       </c>
-      <c r="J16" s="25" t="inlineStr">
+      <c r="J16" s="59" t="inlineStr">
         <is>
           <t>К4 Боли</t>
         </is>
       </c>
-      <c r="K16" s="25" t="inlineStr">
+      <c r="K16" s="59" t="inlineStr">
         <is>
           <t>К5 Дорого</t>
         </is>
       </c>
-      <c r="L16" s="25" t="inlineStr">
+      <c r="L16" s="59" t="inlineStr">
         <is>
           <t>К6 Подумаю</t>
         </is>
       </c>
-      <c r="M16" s="25" t="inlineStr">
+      <c r="M16" s="59" t="inlineStr">
         <is>
           <t>К7 Кейсы</t>
         </is>
       </c>
-      <c r="N16" s="25" t="inlineStr">
+      <c r="N16" s="59" t="inlineStr">
         <is>
           <t>К8 Закрытие</t>
         </is>
       </c>
-      <c r="O16" s="25" t="inlineStr">
+      <c r="O16" s="59" t="inlineStr">
         <is>
           <t>К9 Привет.</t>
         </is>
       </c>
-      <c r="P16" s="25" t="inlineStr">
+      <c r="P16" s="59" t="inlineStr">
         <is>
           <t>К10 Речь</t>
         </is>
       </c>
-      <c r="Q16" s="25" t="inlineStr">
+      <c r="Q16" s="59" t="inlineStr">
         <is>
           <t>К11 Слушан.</t>
         </is>
       </c>
-      <c r="R16" s="25" t="inlineStr">
+      <c r="R16" s="59" t="inlineStr">
         <is>
           <t>К12 Итог</t>
         </is>
       </c>
-      <c r="S16" s="25" t="inlineStr">
+      <c r="S16" s="59" t="inlineStr">
         <is>
           <t>К13 Маржа</t>
         </is>
       </c>
-      <c r="T16" s="25" t="inlineStr">
+      <c r="T16" s="59" t="inlineStr">
         <is>
           <t>Балл /13</t>
         </is>
       </c>
-      <c r="U16" s="25" t="inlineStr">
+      <c r="U16" s="59" t="inlineStr">
         <is>
           <t>Статус ИИ</t>
         </is>
       </c>
-      <c r="V16" s="25" t="inlineStr">
+      <c r="V16" s="59" t="inlineStr">
         <is>
           <t>Сумма в риске, ₽</t>
         </is>
@@ -2727,7 +2739,7 @@
           <t>C-501</t>
         </is>
       </c>
-      <c r="B17" s="60" t="inlineStr">
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>D-101 (ООО Вектор Плюс)</t>
         </is>
@@ -2737,7 +2749,7 @@
           <t>Мельников</t>
         </is>
       </c>
-      <c r="D17" s="67" t="n">
+      <c r="D17" s="68" t="n">
         <v>850000</v>
       </c>
       <c r="E17" s="26" t="inlineStr">
@@ -2750,46 +2762,46 @@
           <t>КП отправлено</t>
         </is>
       </c>
-      <c r="G17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="N17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="O17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="R17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="S17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="T17" s="59">
+      <c r="G17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="R17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" s="60">
         <f>SUM(G17:S17)</f>
         <v/>
       </c>
@@ -2808,7 +2820,7 @@
           <t>C-502</t>
         </is>
       </c>
-      <c r="B18" s="60" t="inlineStr">
+      <c r="B18" s="61" t="inlineStr">
         <is>
           <t>D-104 (ООО Вектор Плюс)</t>
         </is>
@@ -2818,7 +2830,7 @@
           <t>Васильева</t>
         </is>
       </c>
-      <c r="D18" s="67" t="n">
+      <c r="D18" s="68" t="n">
         <v>850000</v>
       </c>
       <c r="E18" s="26" t="inlineStr">
@@ -2831,46 +2843,46 @@
           <t>Переговоры</t>
         </is>
       </c>
-      <c r="G18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="I18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="69" t="n">
+      <c r="G18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="N18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="O18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="R18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="S18" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="T18" s="59">
+      <c r="M18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" s="60">
         <f>SUM(G18:S18)</f>
         <v/>
       </c>
@@ -2889,7 +2901,7 @@
           <t>C-503</t>
         </is>
       </c>
-      <c r="B19" s="60" t="inlineStr">
+      <c r="B19" s="61" t="inlineStr">
         <is>
           <t>D-106 (ООО СнабСервис)</t>
         </is>
@@ -2899,7 +2911,7 @@
           <t>Соколова</t>
         </is>
       </c>
-      <c r="D19" s="67" t="n">
+      <c r="D19" s="68" t="n">
         <v>280000</v>
       </c>
       <c r="E19" s="26" t="inlineStr">
@@ -2912,46 +2924,46 @@
           <t>Встреча/Демо</t>
         </is>
       </c>
-      <c r="G19" s="69" t="n">
+      <c r="G19" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="69" t="n">
+      <c r="H19" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" s="69" t="n">
+      <c r="K19" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M19" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="N19" s="69" t="n">
+      <c r="M19" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="O19" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P19" s="69" t="n">
+      <c r="O19" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="Q19" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="R19" s="69" t="n">
+      <c r="Q19" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="R19" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="S19" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="T19" s="63">
+      <c r="S19" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" s="64">
         <f>SUM(G19:S19)</f>
         <v/>
       </c>
@@ -2960,7 +2972,7 @@
           <t>⚠️ РИСК</t>
         </is>
       </c>
-      <c r="V19" s="61" t="n">
+      <c r="V19" s="62" t="n">
         <v>280000</v>
       </c>
     </row>
@@ -2970,7 +2982,7 @@
           <t>C-504</t>
         </is>
       </c>
-      <c r="B20" s="60" t="inlineStr">
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t>D-107 (ООО ТехноПром)</t>
         </is>
@@ -2980,7 +2992,7 @@
           <t>Соколова</t>
         </is>
       </c>
-      <c r="D20" s="67" t="n">
+      <c r="D20" s="68" t="n">
         <v>150000</v>
       </c>
       <c r="E20" s="26" t="inlineStr">
@@ -2993,46 +3005,46 @@
           <t>Квалификация</t>
         </is>
       </c>
-      <c r="G20" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="69" t="n">
+      <c r="G20" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" s="69" t="n">
+      <c r="K20" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="N20" s="69" t="n">
+      <c r="N20" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="O20" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P20" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="69" t="n">
+      <c r="O20" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P20" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="R20" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="S20" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="T20" s="62">
+      <c r="R20" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="T20" s="63">
         <f>SUM(G20:S20)</f>
         <v/>
       </c>
@@ -3041,7 +3053,7 @@
           <t>⚠️ РИСК</t>
         </is>
       </c>
-      <c r="V20" s="61" t="n">
+      <c r="V20" s="62" t="n">
         <v>150000</v>
       </c>
     </row>
@@ -3051,7 +3063,7 @@
           <t>C-505</t>
         </is>
       </c>
-      <c r="B21" s="60" t="inlineStr">
+      <c r="B21" s="61" t="inlineStr">
         <is>
           <t>D-109 (ООО ПромКомплект)</t>
         </is>
@@ -3061,7 +3073,7 @@
           <t>Ковалев</t>
         </is>
       </c>
-      <c r="D21" s="67" t="n">
+      <c r="D21" s="68" t="n">
         <v>600000</v>
       </c>
       <c r="E21" s="26" t="inlineStr">
@@ -3074,46 +3086,46 @@
           <t>КП отправлено</t>
         </is>
       </c>
-      <c r="G21" s="69" t="n">
+      <c r="G21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="69" t="n">
+      <c r="H21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="69" t="n">
+      <c r="I21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="69" t="n">
+      <c r="J21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="K21" s="69" t="n">
+      <c r="K21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="L21" s="69" t="n">
+      <c r="L21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M21" s="69" t="n">
+      <c r="M21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="N21" s="69" t="n">
+      <c r="N21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="O21" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P21" s="69" t="n">
+      <c r="O21" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="Q21" s="69" t="n">
+      <c r="Q21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="R21" s="69" t="n">
+      <c r="R21" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="S21" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="T21" s="63">
+      <c r="S21" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="T21" s="64">
         <f>SUM(G21:S21)</f>
         <v/>
       </c>
@@ -3122,7 +3134,7 @@
           <t>❌ СЛИВ</t>
         </is>
       </c>
-      <c r="V21" s="61" t="n">
+      <c r="V21" s="62" t="n">
         <v>600000</v>
       </c>
     </row>
@@ -3132,7 +3144,7 @@
           <t>C-506</t>
         </is>
       </c>
-      <c r="B22" s="60" t="inlineStr">
+      <c r="B22" s="61" t="inlineStr">
         <is>
           <t>D-111 (ООО Глобал Инвест)</t>
         </is>
@@ -3142,7 +3154,7 @@
           <t>Мельников</t>
         </is>
       </c>
-      <c r="D22" s="67" t="n">
+      <c r="D22" s="68" t="n">
         <v>3000000</v>
       </c>
       <c r="E22" s="26" t="inlineStr">
@@ -3155,46 +3167,46 @@
           <t>Финальные условия</t>
         </is>
       </c>
-      <c r="G22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="K22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="M22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="N22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="O22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="R22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="S22" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="T22" s="59">
+      <c r="G22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="R22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="T22" s="60">
         <f>SUM(G22:S22)</f>
         <v/>
       </c>
@@ -3213,7 +3225,7 @@
           <t>C-507</t>
         </is>
       </c>
-      <c r="B23" s="60" t="inlineStr">
+      <c r="B23" s="61" t="inlineStr">
         <is>
           <t>D-114 (ООО АльфаТрейд)</t>
         </is>
@@ -3223,7 +3235,7 @@
           <t>Ковалев</t>
         </is>
       </c>
-      <c r="D23" s="67" t="n">
+      <c r="D23" s="68" t="n">
         <v>500000</v>
       </c>
       <c r="E23" s="26" t="inlineStr">
@@ -3236,46 +3248,46 @@
           <t>Дожим договора</t>
         </is>
       </c>
-      <c r="G23" s="69" t="n">
+      <c r="G23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J23" s="69" t="n">
+      <c r="H23" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="69" t="n">
+      <c r="K23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="L23" s="69" t="n">
+      <c r="L23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M23" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="N23" s="69" t="n">
+      <c r="M23" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="O23" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P23" s="69" t="n">
+      <c r="O23" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="Q23" s="69" t="n">
+      <c r="Q23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="R23" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="S23" s="69" t="n">
+      <c r="R23" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="T23" s="63">
+      <c r="T23" s="64">
         <f>SUM(G23:S23)</f>
         <v/>
       </c>
@@ -3284,7 +3296,7 @@
           <t>❌ СЛИВ</t>
         </is>
       </c>
-      <c r="V23" s="61" t="n">
+      <c r="V23" s="62" t="n">
         <v>500000</v>
       </c>
     </row>
@@ -3294,7 +3306,7 @@
           <t>C-508</t>
         </is>
       </c>
-      <c r="B24" s="60" t="inlineStr">
+      <c r="B24" s="61" t="inlineStr">
         <is>
           <t>D-118 (ООО СтройХолдинг)</t>
         </is>
@@ -3304,7 +3316,7 @@
           <t>Попов</t>
         </is>
       </c>
-      <c r="D24" s="67" t="n">
+      <c r="D24" s="68" t="n">
         <v>650000</v>
       </c>
       <c r="E24" s="26" t="inlineStr">
@@ -3317,46 +3329,46 @@
           <t>Входящий лид</t>
         </is>
       </c>
-      <c r="G24" s="69" t="n">
+      <c r="G24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="69" t="n">
+      <c r="H24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="69" t="n">
+      <c r="I24" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="69" t="n">
+      <c r="K24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="L24" s="69" t="n">
+      <c r="L24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M24" s="69" t="n">
+      <c r="M24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="N24" s="69" t="n">
+      <c r="N24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="O24" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P24" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q24" s="69" t="n">
+      <c r="O24" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="R24" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="S24" s="69" t="n">
+      <c r="R24" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="T24" s="63">
+      <c r="T24" s="64">
         <f>SUM(G24:S24)</f>
         <v/>
       </c>
@@ -3365,7 +3377,7 @@
           <t>❌ СЛИВ</t>
         </is>
       </c>
-      <c r="V24" s="61" t="n">
+      <c r="V24" s="62" t="n">
         <v>650000</v>
       </c>
     </row>
@@ -3375,7 +3387,7 @@
           <t>C-509</t>
         </is>
       </c>
-      <c r="B25" s="60" t="inlineStr">
+      <c r="B25" s="61" t="inlineStr">
         <is>
           <t>D-121 (ООО СпецМаш)</t>
         </is>
@@ -3385,7 +3397,7 @@
           <t>Васильева</t>
         </is>
       </c>
-      <c r="D25" s="67" t="n">
+      <c r="D25" s="68" t="n">
         <v>420000</v>
       </c>
       <c r="E25" s="26" t="inlineStr">
@@ -3398,46 +3410,46 @@
           <t>Презентация КП</t>
         </is>
       </c>
-      <c r="G25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="H25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="I25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="L25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="M25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="N25" s="69" t="n">
+      <c r="G25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="N25" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="O25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="R25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="S25" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="T25" s="59">
+      <c r="O25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="R25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="T25" s="60">
         <f>SUM(G25:S25)</f>
         <v/>
       </c>
@@ -3456,7 +3468,7 @@
           <t>C-510</t>
         </is>
       </c>
-      <c r="B26" s="60" t="inlineStr">
+      <c r="B26" s="61" t="inlineStr">
         <is>
           <t>D-125 (ООО МегаТранс)</t>
         </is>
@@ -3466,7 +3478,7 @@
           <t>Попов</t>
         </is>
       </c>
-      <c r="D26" s="67" t="n">
+      <c r="D26" s="68" t="n">
         <v>450000</v>
       </c>
       <c r="E26" s="26" t="inlineStr">
@@ -3479,46 +3491,46 @@
           <t>Квалификация</t>
         </is>
       </c>
-      <c r="G26" s="69" t="n">
+      <c r="G26" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="69" t="n">
+      <c r="H26" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="I26" s="69" t="n">
+      <c r="I26" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="L26" s="69" t="n">
+      <c r="J26" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L26" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M26" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="N26" s="69" t="n">
+      <c r="M26" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="O26" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="P26" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q26" s="69" t="n">
+      <c r="O26" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="P26" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="R26" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="S26" s="69" t="n">
+      <c r="R26" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="T26" s="63">
+      <c r="T26" s="64">
         <f>SUM(G26:S26)</f>
         <v/>
       </c>
@@ -3527,19 +3539,19 @@
           <t>⚠️ РИСК</t>
         </is>
       </c>
-      <c r="V26" s="61" t="n">
+      <c r="V26" s="62" t="n">
         <v>450000</v>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="29" t="inlineStr"/>
-      <c r="B27" s="30" t="inlineStr">
+      <c r="A27" s="30" t="inlineStr">
         <is>
           <t>ИТОГО ПОТЕРЬ И РИСКОВ ПО ЗВОНКАМ:</t>
         </is>
       </c>
-      <c r="C27" s="29" t="inlineStr"/>
-      <c r="D27" s="70">
+      <c r="B27" s="30" t="n"/>
+      <c r="C27" s="30" t="n"/>
+      <c r="D27" s="71">
         <f>SUM(D17:D26)</f>
         <v/>
       </c>
@@ -3558,11 +3570,11 @@
       <c r="Q27" s="29" t="inlineStr"/>
       <c r="R27" s="29" t="inlineStr"/>
       <c r="S27" s="29" t="inlineStr"/>
-      <c r="T27" s="71">
+      <c r="T27" s="72">
         <f>AVERAGE(T17:T26)</f>
         <v/>
       </c>
-      <c r="U27" s="72" t="inlineStr">
+      <c r="U27" s="73" t="inlineStr">
         <is>
           <t>6 сливов</t>
         </is>
@@ -3659,7 +3671,7 @@
           <t>C-505</t>
         </is>
       </c>
-      <c r="B31" s="73" t="inlineStr">
+      <c r="B31" s="74" t="inlineStr">
         <is>
           <t>D-109 (ООО «ПромКомплект»)</t>
         </is>
@@ -3669,39 +3681,39 @@
           <t>Дмитрий Ковалев</t>
         </is>
       </c>
-      <c r="D31" s="61" t="n">
+      <c r="D31" s="62" t="n">
         <v>600000</v>
       </c>
-      <c r="E31" s="74" t="inlineStr">
+      <c r="E31" s="75" t="inlineStr">
         <is>
           <t>Срыв контакта / грубость при цене</t>
         </is>
       </c>
-      <c r="F31" s="74" t="n"/>
-      <c r="G31" s="75" t="inlineStr">
+      <c r="F31" s="75" t="n"/>
+      <c r="G31" s="76" t="inlineStr">
         <is>
           <t>Клиент: «Почему у вас смета на 15% выше рынка?» → Менеджер: «Не знаю, везде всё дорожает. Не устраивает — берите у конкурентов без гарантии»</t>
         </is>
       </c>
-      <c r="H31" s="75" t="n"/>
-      <c r="I31" s="75" t="n"/>
-      <c r="J31" s="75" t="n"/>
-      <c r="K31" s="75" t="n"/>
-      <c r="L31" s="75" t="n"/>
-      <c r="M31" s="75" t="n"/>
-      <c r="N31" s="76" t="inlineStr">
+      <c r="H31" s="76" t="n"/>
+      <c r="I31" s="76" t="n"/>
+      <c r="J31" s="76" t="n"/>
+      <c r="K31" s="76" t="n"/>
+      <c r="L31" s="76" t="n"/>
+      <c r="M31" s="76" t="n"/>
+      <c r="N31" s="77" t="inlineStr">
         <is>
           <t>🚨 Экстренный звонок РОПа ЛПР до 12:00: принести извинения за консультацию, перехватить сделку, дать проект со спец-гарантией 24 мес.</t>
         </is>
       </c>
-      <c r="O31" s="76" t="n"/>
-      <c r="P31" s="76" t="n"/>
-      <c r="Q31" s="76" t="n"/>
-      <c r="R31" s="76" t="n"/>
-      <c r="S31" s="76" t="n"/>
-      <c r="T31" s="76" t="n"/>
-      <c r="U31" s="76" t="n"/>
-      <c r="V31" s="76" t="n"/>
+      <c r="O31" s="77" t="n"/>
+      <c r="P31" s="77" t="n"/>
+      <c r="Q31" s="77" t="n"/>
+      <c r="R31" s="77" t="n"/>
+      <c r="S31" s="77" t="n"/>
+      <c r="T31" s="77" t="n"/>
+      <c r="U31" s="77" t="n"/>
+      <c r="V31" s="77" t="n"/>
     </row>
     <row r="32" ht="54" customHeight="1">
       <c r="A32" s="44" t="inlineStr">
@@ -3709,7 +3721,7 @@
           <t>C-503</t>
         </is>
       </c>
-      <c r="B32" s="73" t="inlineStr">
+      <c r="B32" s="74" t="inlineStr">
         <is>
           <t>D-106 (ООО «СнабСервис»)</t>
         </is>
@@ -3719,39 +3731,39 @@
           <t>Анна Соколова</t>
         </is>
       </c>
-      <c r="D32" s="61" t="n">
+      <c r="D32" s="62" t="n">
         <v>280000</v>
       </c>
-      <c r="E32" s="74" t="inlineStr">
+      <c r="E32" s="75" t="inlineStr">
         <is>
           <t>Слив жесткого Next Step (в никуда)</t>
         </is>
       </c>
-      <c r="F32" s="74" t="n"/>
-      <c r="G32" s="75" t="inlineStr">
+      <c r="F32" s="75" t="n"/>
+      <c r="G32" s="76" t="inlineStr">
         <is>
           <t>Менеджер: «Я вам КП на почту сбросила, посмотрите когда время будет». Клиент: «Хорошо, если что наберу»</t>
         </is>
       </c>
-      <c r="H32" s="75" t="n"/>
-      <c r="I32" s="75" t="n"/>
-      <c r="J32" s="75" t="n"/>
-      <c r="K32" s="75" t="n"/>
-      <c r="L32" s="75" t="n"/>
-      <c r="M32" s="75" t="n"/>
-      <c r="N32" s="76" t="inlineStr">
+      <c r="H32" s="76" t="n"/>
+      <c r="I32" s="76" t="n"/>
+      <c r="J32" s="76" t="n"/>
+      <c r="K32" s="76" t="n"/>
+      <c r="L32" s="76" t="n"/>
+      <c r="M32" s="76" t="n"/>
+      <c r="N32" s="77" t="inlineStr">
         <is>
           <t>Направить клиенту в WhatsApp 2 конкретных слота встречи (сегодня 16:00 / завтра 11:30) с демонстрацией интеграции с CRM.</t>
         </is>
       </c>
-      <c r="O32" s="76" t="n"/>
-      <c r="P32" s="76" t="n"/>
-      <c r="Q32" s="76" t="n"/>
-      <c r="R32" s="76" t="n"/>
-      <c r="S32" s="76" t="n"/>
-      <c r="T32" s="76" t="n"/>
-      <c r="U32" s="76" t="n"/>
-      <c r="V32" s="76" t="n"/>
+      <c r="O32" s="77" t="n"/>
+      <c r="P32" s="77" t="n"/>
+      <c r="Q32" s="77" t="n"/>
+      <c r="R32" s="77" t="n"/>
+      <c r="S32" s="77" t="n"/>
+      <c r="T32" s="77" t="n"/>
+      <c r="U32" s="77" t="n"/>
+      <c r="V32" s="77" t="n"/>
     </row>
     <row r="33" ht="54" customHeight="1">
       <c r="A33" s="44" t="inlineStr">
@@ -3759,7 +3771,7 @@
           <t>C-507</t>
         </is>
       </c>
-      <c r="B33" s="73" t="inlineStr">
+      <c r="B33" s="74" t="inlineStr">
         <is>
           <t>D-114 (ООО «АльфаТрейд»)</t>
         </is>
@@ -3769,39 +3781,39 @@
           <t>Дмитрий Ковалев</t>
         </is>
       </c>
-      <c r="D33" s="61" t="n">
+      <c r="D33" s="62" t="n">
         <v>500000</v>
       </c>
-      <c r="E33" s="74" t="inlineStr">
+      <c r="E33" s="75" t="inlineStr">
         <is>
           <t>Необоснованная скидка вместо ценности</t>
         </is>
       </c>
-      <c r="F33" s="74" t="n"/>
-      <c r="G33" s="75" t="inlineStr">
+      <c r="F33" s="75" t="n"/>
+      <c r="G33" s="76" t="inlineStr">
         <is>
           <t>Клиент: «У нас бюджет строго ограничен». Менеджер: «Ну ладно, согласую вам скидку 10% прямо сейчас»</t>
         </is>
       </c>
-      <c r="H33" s="75" t="n"/>
-      <c r="I33" s="75" t="n"/>
-      <c r="J33" s="75" t="n"/>
-      <c r="K33" s="75" t="n"/>
-      <c r="L33" s="75" t="n"/>
-      <c r="M33" s="75" t="n"/>
-      <c r="N33" s="76" t="inlineStr">
+      <c r="H33" s="76" t="n"/>
+      <c r="I33" s="76" t="n"/>
+      <c r="J33" s="76" t="n"/>
+      <c r="K33" s="76" t="n"/>
+      <c r="L33" s="76" t="n"/>
+      <c r="M33" s="76" t="n"/>
+      <c r="N33" s="77" t="inlineStr">
         <is>
           <t>Заблокировать выставление счета со скидкой в CRM. РОПу пересогласовать условия: скидка 5% только в обмен на 100% предоплату за 24ч.</t>
         </is>
       </c>
-      <c r="O33" s="76" t="n"/>
-      <c r="P33" s="76" t="n"/>
-      <c r="Q33" s="76" t="n"/>
-      <c r="R33" s="76" t="n"/>
-      <c r="S33" s="76" t="n"/>
-      <c r="T33" s="76" t="n"/>
-      <c r="U33" s="76" t="n"/>
-      <c r="V33" s="76" t="n"/>
+      <c r="O33" s="77" t="n"/>
+      <c r="P33" s="77" t="n"/>
+      <c r="Q33" s="77" t="n"/>
+      <c r="R33" s="77" t="n"/>
+      <c r="S33" s="77" t="n"/>
+      <c r="T33" s="77" t="n"/>
+      <c r="U33" s="77" t="n"/>
+      <c r="V33" s="77" t="n"/>
     </row>
     <row r="34" ht="54" customHeight="1">
       <c r="A34" s="44" t="inlineStr">
@@ -3809,7 +3821,7 @@
           <t>C-508</t>
         </is>
       </c>
-      <c r="B34" s="73" t="inlineStr">
+      <c r="B34" s="74" t="inlineStr">
         <is>
           <t>D-118 (ООО «СтройХолдинг»)</t>
         </is>
@@ -3819,39 +3831,39 @@
           <t>Иван Попов</t>
         </is>
       </c>
-      <c r="D34" s="61" t="n">
+      <c r="D34" s="62" t="n">
         <v>650000</v>
       </c>
-      <c r="E34" s="74" t="inlineStr">
+      <c r="E34" s="75" t="inlineStr">
         <is>
           <t>Слив возражения «Я подумаю»</t>
         </is>
       </c>
-      <c r="F34" s="74" t="n"/>
-      <c r="G34" s="75" t="inlineStr">
+      <c r="F34" s="75" t="n"/>
+      <c r="G34" s="76" t="inlineStr">
         <is>
           <t>Клиент: «Нам нужно всё обдумать и посоветоваться с руководством». Менеджер: «Да, конечно, думайте» (повесил трубку)</t>
         </is>
       </c>
-      <c r="H34" s="75" t="n"/>
-      <c r="I34" s="75" t="n"/>
-      <c r="J34" s="75" t="n"/>
-      <c r="K34" s="75" t="n"/>
-      <c r="L34" s="75" t="n"/>
-      <c r="M34" s="75" t="n"/>
-      <c r="N34" s="76" t="inlineStr">
+      <c r="H34" s="76" t="n"/>
+      <c r="I34" s="76" t="n"/>
+      <c r="J34" s="76" t="n"/>
+      <c r="K34" s="76" t="n"/>
+      <c r="L34" s="76" t="n"/>
+      <c r="M34" s="76" t="n"/>
+      <c r="N34" s="77" t="inlineStr">
         <is>
           <t>Передать лида старшему КАМу. Отправить в WhatsApp отраслевой кейс с аналогичным объектом и окупаемостью за 21 день.</t>
         </is>
       </c>
-      <c r="O34" s="76" t="n"/>
-      <c r="P34" s="76" t="n"/>
-      <c r="Q34" s="76" t="n"/>
-      <c r="R34" s="76" t="n"/>
-      <c r="S34" s="76" t="n"/>
-      <c r="T34" s="76" t="n"/>
-      <c r="U34" s="76" t="n"/>
-      <c r="V34" s="76" t="n"/>
+      <c r="O34" s="77" t="n"/>
+      <c r="P34" s="77" t="n"/>
+      <c r="Q34" s="77" t="n"/>
+      <c r="R34" s="77" t="n"/>
+      <c r="S34" s="77" t="n"/>
+      <c r="T34" s="77" t="n"/>
+      <c r="U34" s="77" t="n"/>
+      <c r="V34" s="77" t="n"/>
     </row>
     <row r="35" ht="54" customHeight="1">
       <c r="A35" s="44" t="inlineStr">
@@ -3859,7 +3871,7 @@
           <t>C-510</t>
         </is>
       </c>
-      <c r="B35" s="73" t="inlineStr">
+      <c r="B35" s="74" t="inlineStr">
         <is>
           <t>D-125 (ООО «МегаТранс»)</t>
         </is>
@@ -3869,39 +3881,39 @@
           <t>Иван Попов</t>
         </is>
       </c>
-      <c r="D35" s="61" t="n">
+      <c r="D35" s="62" t="n">
         <v>450000</v>
       </c>
-      <c r="E35" s="74" t="inlineStr">
+      <c r="E35" s="75" t="inlineStr">
         <is>
           <t>Режим автоответчика, не выявлен ЛПР</t>
         </is>
       </c>
-      <c r="F35" s="74" t="n"/>
-      <c r="G35" s="75" t="inlineStr">
+      <c r="F35" s="75" t="n"/>
+      <c r="G35" s="76" t="inlineStr">
         <is>
           <t>Менеджер 5 минут зачитывал прайс-лист секретарю, не спросив, кто принимает решение по закупкам</t>
         </is>
       </c>
-      <c r="H35" s="75" t="n"/>
-      <c r="I35" s="75" t="n"/>
-      <c r="J35" s="75" t="n"/>
-      <c r="K35" s="75" t="n"/>
-      <c r="L35" s="75" t="n"/>
-      <c r="M35" s="75" t="n"/>
-      <c r="N35" s="76" t="inlineStr">
+      <c r="H35" s="76" t="n"/>
+      <c r="I35" s="76" t="n"/>
+      <c r="J35" s="76" t="n"/>
+      <c r="K35" s="76" t="n"/>
+      <c r="L35" s="76" t="n"/>
+      <c r="M35" s="76" t="n"/>
+      <c r="N35" s="77" t="inlineStr">
         <is>
           <t>Разбор на летучке: регламент квалификации BANT. Назначить повторный звонок с прямым выходом на генерального директора.</t>
         </is>
       </c>
-      <c r="O35" s="76" t="n"/>
-      <c r="P35" s="76" t="n"/>
-      <c r="Q35" s="76" t="n"/>
-      <c r="R35" s="76" t="n"/>
-      <c r="S35" s="76" t="n"/>
-      <c r="T35" s="76" t="n"/>
-      <c r="U35" s="76" t="n"/>
-      <c r="V35" s="76" t="n"/>
+      <c r="O35" s="77" t="n"/>
+      <c r="P35" s="77" t="n"/>
+      <c r="Q35" s="77" t="n"/>
+      <c r="R35" s="77" t="n"/>
+      <c r="S35" s="77" t="n"/>
+      <c r="T35" s="77" t="n"/>
+      <c r="U35" s="77" t="n"/>
+      <c r="V35" s="77" t="n"/>
     </row>
     <row r="36" ht="12" customHeight="1"/>
     <row r="37" ht="24" customHeight="1">
@@ -4010,29 +4022,29 @@
       </c>
       <c r="F39" s="27" t="n"/>
       <c r="G39" s="27" t="n"/>
-      <c r="H39" s="77" t="inlineStr">
+      <c r="H39" s="78" t="inlineStr">
         <is>
           <t>«Я вам перезвоню на днях», «Подумайте, наберите», отпускание без времени</t>
         </is>
       </c>
-      <c r="I39" s="77" t="n"/>
-      <c r="J39" s="77" t="n"/>
-      <c r="K39" s="77" t="n"/>
-      <c r="L39" s="77" t="n"/>
-      <c r="M39" s="73" t="inlineStr">
+      <c r="I39" s="78" t="n"/>
+      <c r="J39" s="78" t="n"/>
+      <c r="K39" s="78" t="n"/>
+      <c r="L39" s="78" t="n"/>
+      <c r="M39" s="74" t="inlineStr">
         <is>
           <t>Внедрить обязательный вопрос в конце диалога: «Во вторник в 14:30 или в среду в 11:00 удобно?»</t>
         </is>
       </c>
-      <c r="N39" s="73" t="n"/>
-      <c r="O39" s="73" t="n"/>
-      <c r="P39" s="73" t="n"/>
-      <c r="Q39" s="73" t="n"/>
-      <c r="R39" s="73" t="n"/>
-      <c r="S39" s="73" t="n"/>
-      <c r="T39" s="73" t="n"/>
-      <c r="U39" s="73" t="n"/>
-      <c r="V39" s="73" t="n"/>
+      <c r="N39" s="74" t="n"/>
+      <c r="O39" s="74" t="n"/>
+      <c r="P39" s="74" t="n"/>
+      <c r="Q39" s="74" t="n"/>
+      <c r="R39" s="74" t="n"/>
+      <c r="S39" s="74" t="n"/>
+      <c r="T39" s="74" t="n"/>
+      <c r="U39" s="74" t="n"/>
+      <c r="V39" s="74" t="n"/>
     </row>
     <row r="40" ht="34" customHeight="1">
       <c r="A40" s="26" t="n">
@@ -4060,29 +4072,29 @@
       </c>
       <c r="F40" s="27" t="n"/>
       <c r="G40" s="27" t="n"/>
-      <c r="H40" s="77" t="inlineStr">
+      <c r="H40" s="78" t="inlineStr">
         <is>
           <t>Клиент задает все вопросы сам, менеджер только отвечает короткими репликами</t>
         </is>
       </c>
-      <c r="I40" s="77" t="n"/>
-      <c r="J40" s="77" t="n"/>
-      <c r="K40" s="77" t="n"/>
-      <c r="L40" s="77" t="n"/>
-      <c r="M40" s="73" t="inlineStr">
+      <c r="I40" s="78" t="n"/>
+      <c r="J40" s="78" t="n"/>
+      <c r="K40" s="78" t="n"/>
+      <c r="L40" s="78" t="n"/>
+      <c r="M40" s="74" t="inlineStr">
         <is>
           <t>Правило «Ответ + Встречный вопрос». Завершать каждую реплику квалифицирующим вопросом.</t>
         </is>
       </c>
-      <c r="N40" s="73" t="n"/>
-      <c r="O40" s="73" t="n"/>
-      <c r="P40" s="73" t="n"/>
-      <c r="Q40" s="73" t="n"/>
-      <c r="R40" s="73" t="n"/>
-      <c r="S40" s="73" t="n"/>
-      <c r="T40" s="73" t="n"/>
-      <c r="U40" s="73" t="n"/>
-      <c r="V40" s="73" t="n"/>
+      <c r="N40" s="74" t="n"/>
+      <c r="O40" s="74" t="n"/>
+      <c r="P40" s="74" t="n"/>
+      <c r="Q40" s="74" t="n"/>
+      <c r="R40" s="74" t="n"/>
+      <c r="S40" s="74" t="n"/>
+      <c r="T40" s="74" t="n"/>
+      <c r="U40" s="74" t="n"/>
+      <c r="V40" s="74" t="n"/>
     </row>
     <row r="41" ht="34" customHeight="1">
       <c r="A41" s="26" t="n">
@@ -4110,29 +4122,29 @@
       </c>
       <c r="F41" s="27" t="n"/>
       <c r="G41" s="27" t="n"/>
-      <c r="H41" s="77" t="inlineStr">
+      <c r="H41" s="78" t="inlineStr">
         <is>
           <t>Трата 40 минут на презентацию инженеру или секретарю без полномочий подписания</t>
         </is>
       </c>
-      <c r="I41" s="77" t="n"/>
-      <c r="J41" s="77" t="n"/>
-      <c r="K41" s="77" t="n"/>
-      <c r="L41" s="77" t="n"/>
-      <c r="M41" s="73" t="inlineStr">
+      <c r="I41" s="78" t="n"/>
+      <c r="J41" s="78" t="n"/>
+      <c r="K41" s="78" t="n"/>
+      <c r="L41" s="78" t="n"/>
+      <c r="M41" s="74" t="inlineStr">
         <is>
           <t>«Кто кроме вас участвует в согласовании проекта и утверждении финансового бюджета?»</t>
         </is>
       </c>
-      <c r="N41" s="73" t="n"/>
-      <c r="O41" s="73" t="n"/>
-      <c r="P41" s="73" t="n"/>
-      <c r="Q41" s="73" t="n"/>
-      <c r="R41" s="73" t="n"/>
-      <c r="S41" s="73" t="n"/>
-      <c r="T41" s="73" t="n"/>
-      <c r="U41" s="73" t="n"/>
-      <c r="V41" s="73" t="n"/>
+      <c r="N41" s="74" t="n"/>
+      <c r="O41" s="74" t="n"/>
+      <c r="P41" s="74" t="n"/>
+      <c r="Q41" s="74" t="n"/>
+      <c r="R41" s="74" t="n"/>
+      <c r="S41" s="74" t="n"/>
+      <c r="T41" s="74" t="n"/>
+      <c r="U41" s="74" t="n"/>
+      <c r="V41" s="74" t="n"/>
     </row>
     <row r="42" ht="34" customHeight="1">
       <c r="A42" s="26" t="n">
@@ -4160,29 +4172,29 @@
       </c>
       <c r="F42" s="27" t="n"/>
       <c r="G42" s="27" t="n"/>
-      <c r="H42" s="77" t="inlineStr">
+      <c r="H42" s="78" t="inlineStr">
         <is>
           <t>Менеджер сразу начинает презентовать продукт, не узнав текущую ситуацию клиента</t>
         </is>
       </c>
-      <c r="I42" s="77" t="n"/>
-      <c r="J42" s="77" t="n"/>
-      <c r="K42" s="77" t="n"/>
-      <c r="L42" s="77" t="n"/>
-      <c r="M42" s="73" t="inlineStr">
+      <c r="I42" s="78" t="n"/>
+      <c r="J42" s="78" t="n"/>
+      <c r="K42" s="78" t="n"/>
+      <c r="L42" s="78" t="n"/>
+      <c r="M42" s="74" t="inlineStr">
         <is>
           <t>Сначала диагностика по методологии SPIN/BANT, затем презентация под конкретную боль.</t>
         </is>
       </c>
-      <c r="N42" s="73" t="n"/>
-      <c r="O42" s="73" t="n"/>
-      <c r="P42" s="73" t="n"/>
-      <c r="Q42" s="73" t="n"/>
-      <c r="R42" s="73" t="n"/>
-      <c r="S42" s="73" t="n"/>
-      <c r="T42" s="73" t="n"/>
-      <c r="U42" s="73" t="n"/>
-      <c r="V42" s="73" t="n"/>
+      <c r="N42" s="74" t="n"/>
+      <c r="O42" s="74" t="n"/>
+      <c r="P42" s="74" t="n"/>
+      <c r="Q42" s="74" t="n"/>
+      <c r="R42" s="74" t="n"/>
+      <c r="S42" s="74" t="n"/>
+      <c r="T42" s="74" t="n"/>
+      <c r="U42" s="74" t="n"/>
+      <c r="V42" s="74" t="n"/>
     </row>
     <row r="43" ht="34" customHeight="1">
       <c r="A43" s="26" t="n">
@@ -4210,29 +4222,29 @@
       </c>
       <c r="F43" s="27" t="n"/>
       <c r="G43" s="27" t="n"/>
-      <c r="H43" s="77" t="inlineStr">
+      <c r="H43" s="78" t="inlineStr">
         <is>
           <t>Моментальная скидка при первом сомнении клиента или согласие («Да, у нас недешево»)</t>
         </is>
       </c>
-      <c r="I43" s="77" t="n"/>
-      <c r="J43" s="77" t="n"/>
-      <c r="K43" s="77" t="n"/>
-      <c r="L43" s="77" t="n"/>
-      <c r="M43" s="73" t="inlineStr">
+      <c r="I43" s="78" t="n"/>
+      <c r="J43" s="78" t="n"/>
+      <c r="K43" s="78" t="n"/>
+      <c r="L43" s="78" t="n"/>
+      <c r="M43" s="74" t="inlineStr">
         <is>
           <t>Обосновать окупаемость: показать, сколько клиент теряет каждый день без внедрения решения.</t>
         </is>
       </c>
-      <c r="N43" s="73" t="n"/>
-      <c r="O43" s="73" t="n"/>
-      <c r="P43" s="73" t="n"/>
-      <c r="Q43" s="73" t="n"/>
-      <c r="R43" s="73" t="n"/>
-      <c r="S43" s="73" t="n"/>
-      <c r="T43" s="73" t="n"/>
-      <c r="U43" s="73" t="n"/>
-      <c r="V43" s="73" t="n"/>
+      <c r="N43" s="74" t="n"/>
+      <c r="O43" s="74" t="n"/>
+      <c r="P43" s="74" t="n"/>
+      <c r="Q43" s="74" t="n"/>
+      <c r="R43" s="74" t="n"/>
+      <c r="S43" s="74" t="n"/>
+      <c r="T43" s="74" t="n"/>
+      <c r="U43" s="74" t="n"/>
+      <c r="V43" s="74" t="n"/>
     </row>
     <row r="44" ht="34" customHeight="1">
       <c r="A44" s="26" t="n">
@@ -4260,29 +4272,29 @@
       </c>
       <c r="F44" s="27" t="n"/>
       <c r="G44" s="27" t="n"/>
-      <c r="H44" s="77" t="inlineStr">
+      <c r="H44" s="78" t="inlineStr">
         <is>
           <t>«Хорошо, думайте, ждем вашего звонка», завершение диалога на неопределенности</t>
         </is>
       </c>
-      <c r="I44" s="77" t="n"/>
-      <c r="J44" s="77" t="n"/>
-      <c r="K44" s="77" t="n"/>
-      <c r="L44" s="77" t="n"/>
-      <c r="M44" s="73" t="inlineStr">
+      <c r="I44" s="78" t="n"/>
+      <c r="J44" s="78" t="n"/>
+      <c r="K44" s="78" t="n"/>
+      <c r="L44" s="78" t="n"/>
+      <c r="M44" s="74" t="inlineStr">
         <is>
           <t>«Алексей, обычно говорят 'подумаю', когда смущает цена или функционал. Что именно из этого?»</t>
         </is>
       </c>
-      <c r="N44" s="73" t="n"/>
-      <c r="O44" s="73" t="n"/>
-      <c r="P44" s="73" t="n"/>
-      <c r="Q44" s="73" t="n"/>
-      <c r="R44" s="73" t="n"/>
-      <c r="S44" s="73" t="n"/>
-      <c r="T44" s="73" t="n"/>
-      <c r="U44" s="73" t="n"/>
-      <c r="V44" s="73" t="n"/>
+      <c r="N44" s="74" t="n"/>
+      <c r="O44" s="74" t="n"/>
+      <c r="P44" s="74" t="n"/>
+      <c r="Q44" s="74" t="n"/>
+      <c r="R44" s="74" t="n"/>
+      <c r="S44" s="74" t="n"/>
+      <c r="T44" s="74" t="n"/>
+      <c r="U44" s="74" t="n"/>
+      <c r="V44" s="74" t="n"/>
     </row>
     <row r="45" ht="34" customHeight="1">
       <c r="A45" s="26" t="n">
@@ -4310,29 +4322,29 @@
       </c>
       <c r="F45" s="27" t="n"/>
       <c r="G45" s="27" t="n"/>
-      <c r="H45" s="77" t="inlineStr">
+      <c r="H45" s="78" t="inlineStr">
         <is>
           <t>Абстрактные слова «мы надежные», «у нас высокое качество» без конкретных фактов</t>
         </is>
       </c>
-      <c r="I45" s="77" t="n"/>
-      <c r="J45" s="77" t="n"/>
-      <c r="K45" s="77" t="n"/>
-      <c r="L45" s="77" t="n"/>
-      <c r="M45" s="73" t="inlineStr">
+      <c r="I45" s="78" t="n"/>
+      <c r="J45" s="78" t="n"/>
+      <c r="K45" s="78" t="n"/>
+      <c r="L45" s="78" t="n"/>
+      <c r="M45" s="74" t="inlineStr">
         <is>
           <t>Показать схожий кейс из отрасли клиента: «Для завода X мы сократили потери на 1.4 млн ₽ за 21 день».</t>
         </is>
       </c>
-      <c r="N45" s="73" t="n"/>
-      <c r="O45" s="73" t="n"/>
-      <c r="P45" s="73" t="n"/>
-      <c r="Q45" s="73" t="n"/>
-      <c r="R45" s="73" t="n"/>
-      <c r="S45" s="73" t="n"/>
-      <c r="T45" s="73" t="n"/>
-      <c r="U45" s="73" t="n"/>
-      <c r="V45" s="73" t="n"/>
+      <c r="N45" s="74" t="n"/>
+      <c r="O45" s="74" t="n"/>
+      <c r="P45" s="74" t="n"/>
+      <c r="Q45" s="74" t="n"/>
+      <c r="R45" s="74" t="n"/>
+      <c r="S45" s="74" t="n"/>
+      <c r="T45" s="74" t="n"/>
+      <c r="U45" s="74" t="n"/>
+      <c r="V45" s="74" t="n"/>
     </row>
     <row r="46" ht="34" customHeight="1">
       <c r="A46" s="26" t="n">
@@ -4360,29 +4372,29 @@
       </c>
       <c r="F46" s="27" t="n"/>
       <c r="G46" s="27" t="n"/>
-      <c r="H46" s="77" t="inlineStr">
+      <c r="H46" s="78" t="inlineStr">
         <is>
           <t>Разговор закончился тепло, но менеджер не предложил сделать следующий шаг к оплате</t>
         </is>
       </c>
-      <c r="I46" s="77" t="n"/>
-      <c r="J46" s="77" t="n"/>
-      <c r="K46" s="77" t="n"/>
-      <c r="L46" s="77" t="n"/>
-      <c r="M46" s="73" t="inlineStr">
+      <c r="I46" s="78" t="n"/>
+      <c r="J46" s="78" t="n"/>
+      <c r="K46" s="78" t="n"/>
+      <c r="L46" s="78" t="n"/>
+      <c r="M46" s="74" t="inlineStr">
         <is>
           <t>«Если все параметры подходят, предлагаю сегодня запустить пилот. Куда отправить договор?»</t>
         </is>
       </c>
-      <c r="N46" s="73" t="n"/>
-      <c r="O46" s="73" t="n"/>
-      <c r="P46" s="73" t="n"/>
-      <c r="Q46" s="73" t="n"/>
-      <c r="R46" s="73" t="n"/>
-      <c r="S46" s="73" t="n"/>
-      <c r="T46" s="73" t="n"/>
-      <c r="U46" s="73" t="n"/>
-      <c r="V46" s="73" t="n"/>
+      <c r="N46" s="74" t="n"/>
+      <c r="O46" s="74" t="n"/>
+      <c r="P46" s="74" t="n"/>
+      <c r="Q46" s="74" t="n"/>
+      <c r="R46" s="74" t="n"/>
+      <c r="S46" s="74" t="n"/>
+      <c r="T46" s="74" t="n"/>
+      <c r="U46" s="74" t="n"/>
+      <c r="V46" s="74" t="n"/>
     </row>
     <row r="47" ht="34" customHeight="1">
       <c r="A47" s="26" t="n">
@@ -4398,7 +4410,7 @@
           <t>0.8x</t>
         </is>
       </c>
-      <c r="D47" s="78" t="inlineStr">
+      <c r="D47" s="79" t="inlineStr">
         <is>
           <t>🟢 P2 (Стандарт)</t>
         </is>
@@ -4410,29 +4422,29 @@
       </c>
       <c r="F47" s="27" t="n"/>
       <c r="G47" s="27" t="n"/>
-      <c r="H47" s="77" t="inlineStr">
+      <c r="H47" s="78" t="inlineStr">
         <is>
           <t>Невнятное приветствие, вопрос «Вам удобно говорить?» без обозначения повестки</t>
         </is>
       </c>
-      <c r="I47" s="77" t="n"/>
-      <c r="J47" s="77" t="n"/>
-      <c r="K47" s="77" t="n"/>
-      <c r="L47" s="77" t="n"/>
-      <c r="M47" s="73" t="inlineStr">
+      <c r="I47" s="78" t="n"/>
+      <c r="J47" s="78" t="n"/>
+      <c r="K47" s="78" t="n"/>
+      <c r="L47" s="78" t="n"/>
+      <c r="M47" s="74" t="inlineStr">
         <is>
           <t>«Добрый день! Дмитрий, компания RevOps. Звоню по вашей заявке на аудит воронки. Уделите 5 минут?»</t>
         </is>
       </c>
-      <c r="N47" s="73" t="n"/>
-      <c r="O47" s="73" t="n"/>
-      <c r="P47" s="73" t="n"/>
-      <c r="Q47" s="73" t="n"/>
-      <c r="R47" s="73" t="n"/>
-      <c r="S47" s="73" t="n"/>
-      <c r="T47" s="73" t="n"/>
-      <c r="U47" s="73" t="n"/>
-      <c r="V47" s="73" t="n"/>
+      <c r="N47" s="74" t="n"/>
+      <c r="O47" s="74" t="n"/>
+      <c r="P47" s="74" t="n"/>
+      <c r="Q47" s="74" t="n"/>
+      <c r="R47" s="74" t="n"/>
+      <c r="S47" s="74" t="n"/>
+      <c r="T47" s="74" t="n"/>
+      <c r="U47" s="74" t="n"/>
+      <c r="V47" s="74" t="n"/>
     </row>
     <row r="48" ht="34" customHeight="1">
       <c r="A48" s="26" t="n">
@@ -4448,7 +4460,7 @@
           <t>0.8x</t>
         </is>
       </c>
-      <c r="D48" s="78" t="inlineStr">
+      <c r="D48" s="79" t="inlineStr">
         <is>
           <t>🟢 P2 (Стандарт)</t>
         </is>
@@ -4460,29 +4472,29 @@
       </c>
       <c r="F48" s="27" t="n"/>
       <c r="G48" s="27" t="n"/>
-      <c r="H48" s="77" t="inlineStr">
+      <c r="H48" s="78" t="inlineStr">
         <is>
           <t>Дрожащий голос при озвучивании чека, слова сомнения («может быть», «наверное»)</t>
         </is>
       </c>
-      <c r="I48" s="77" t="n"/>
-      <c r="J48" s="77" t="n"/>
-      <c r="K48" s="77" t="n"/>
-      <c r="L48" s="77" t="n"/>
-      <c r="M48" s="73" t="inlineStr">
+      <c r="I48" s="78" t="n"/>
+      <c r="J48" s="78" t="n"/>
+      <c r="K48" s="78" t="n"/>
+      <c r="L48" s="78" t="n"/>
+      <c r="M48" s="74" t="inlineStr">
         <is>
           <t>Отработать блок цены на тренажере: уверенная пауза после озвучивания стоимости.</t>
         </is>
       </c>
-      <c r="N48" s="73" t="n"/>
-      <c r="O48" s="73" t="n"/>
-      <c r="P48" s="73" t="n"/>
-      <c r="Q48" s="73" t="n"/>
-      <c r="R48" s="73" t="n"/>
-      <c r="S48" s="73" t="n"/>
-      <c r="T48" s="73" t="n"/>
-      <c r="U48" s="73" t="n"/>
-      <c r="V48" s="73" t="n"/>
+      <c r="N48" s="74" t="n"/>
+      <c r="O48" s="74" t="n"/>
+      <c r="P48" s="74" t="n"/>
+      <c r="Q48" s="74" t="n"/>
+      <c r="R48" s="74" t="n"/>
+      <c r="S48" s="74" t="n"/>
+      <c r="T48" s="74" t="n"/>
+      <c r="U48" s="74" t="n"/>
+      <c r="V48" s="74" t="n"/>
     </row>
     <row r="49" ht="34" customHeight="1">
       <c r="A49" s="26" t="n">
@@ -4510,29 +4522,29 @@
       </c>
       <c r="F49" s="27" t="n"/>
       <c r="G49" s="27" t="n"/>
-      <c r="H49" s="77" t="inlineStr">
+      <c r="H49" s="78" t="inlineStr">
         <is>
           <t>Монолог менеджера &gt; 70% времени: клиент молчит и теряет фокус внимания</t>
         </is>
       </c>
-      <c r="I49" s="77" t="n"/>
-      <c r="J49" s="77" t="n"/>
-      <c r="K49" s="77" t="n"/>
-      <c r="L49" s="77" t="n"/>
-      <c r="M49" s="73" t="inlineStr">
+      <c r="I49" s="78" t="n"/>
+      <c r="J49" s="78" t="n"/>
+      <c r="K49" s="78" t="n"/>
+      <c r="L49" s="78" t="n"/>
+      <c r="M49" s="74" t="inlineStr">
         <is>
           <t>Держать баланс 50/50. Задавать открытые вопросы и давать клиенту выговориться о проблеме.</t>
         </is>
       </c>
-      <c r="N49" s="73" t="n"/>
-      <c r="O49" s="73" t="n"/>
-      <c r="P49" s="73" t="n"/>
-      <c r="Q49" s="73" t="n"/>
-      <c r="R49" s="73" t="n"/>
-      <c r="S49" s="73" t="n"/>
-      <c r="T49" s="73" t="n"/>
-      <c r="U49" s="73" t="n"/>
-      <c r="V49" s="73" t="n"/>
+      <c r="N49" s="74" t="n"/>
+      <c r="O49" s="74" t="n"/>
+      <c r="P49" s="74" t="n"/>
+      <c r="Q49" s="74" t="n"/>
+      <c r="R49" s="74" t="n"/>
+      <c r="S49" s="74" t="n"/>
+      <c r="T49" s="74" t="n"/>
+      <c r="U49" s="74" t="n"/>
+      <c r="V49" s="74" t="n"/>
     </row>
     <row r="50" ht="34" customHeight="1">
       <c r="A50" s="26" t="n">
@@ -4548,7 +4560,7 @@
           <t>1.0x</t>
         </is>
       </c>
-      <c r="D50" s="78" t="inlineStr">
+      <c r="D50" s="79" t="inlineStr">
         <is>
           <t>🟢 P2 (Стандарт)</t>
         </is>
@@ -4560,29 +4572,29 @@
       </c>
       <c r="F50" s="27" t="n"/>
       <c r="G50" s="27" t="n"/>
-      <c r="H50" s="77" t="inlineStr">
+      <c r="H50" s="78" t="inlineStr">
         <is>
           <t>Диалог оборвался, у клиента и менеджера разное понимание следующих действий</t>
         </is>
       </c>
-      <c r="I50" s="77" t="n"/>
-      <c r="J50" s="77" t="n"/>
-      <c r="K50" s="77" t="n"/>
-      <c r="L50" s="77" t="n"/>
-      <c r="M50" s="73" t="inlineStr">
+      <c r="I50" s="78" t="n"/>
+      <c r="J50" s="78" t="n"/>
+      <c r="K50" s="78" t="n"/>
+      <c r="L50" s="78" t="n"/>
+      <c r="M50" s="74" t="inlineStr">
         <is>
           <t>«Итак, резюмирую: я отправляю КП в WhatsApp до 15:00, а завтра в 11:00 мы созваниваемся по условиям».</t>
         </is>
       </c>
-      <c r="N50" s="73" t="n"/>
-      <c r="O50" s="73" t="n"/>
-      <c r="P50" s="73" t="n"/>
-      <c r="Q50" s="73" t="n"/>
-      <c r="R50" s="73" t="n"/>
-      <c r="S50" s="73" t="n"/>
-      <c r="T50" s="73" t="n"/>
-      <c r="U50" s="73" t="n"/>
-      <c r="V50" s="73" t="n"/>
+      <c r="N50" s="74" t="n"/>
+      <c r="O50" s="74" t="n"/>
+      <c r="P50" s="74" t="n"/>
+      <c r="Q50" s="74" t="n"/>
+      <c r="R50" s="74" t="n"/>
+      <c r="S50" s="74" t="n"/>
+      <c r="T50" s="74" t="n"/>
+      <c r="U50" s="74" t="n"/>
+      <c r="V50" s="74" t="n"/>
     </row>
     <row r="51" ht="34" customHeight="1">
       <c r="A51" s="26" t="n">
@@ -4610,29 +4622,29 @@
       </c>
       <c r="F51" s="27" t="n"/>
       <c r="G51" s="27" t="n"/>
-      <c r="H51" s="77" t="inlineStr">
+      <c r="H51" s="78" t="inlineStr">
         <is>
           <t>Раздача скидок из маржи компании без требования 100% предоплаты или большего объема</t>
         </is>
       </c>
-      <c r="I51" s="77" t="n"/>
-      <c r="J51" s="77" t="n"/>
-      <c r="K51" s="77" t="n"/>
-      <c r="L51" s="77" t="n"/>
-      <c r="M51" s="73" t="inlineStr">
+      <c r="I51" s="78" t="n"/>
+      <c r="J51" s="78" t="n"/>
+      <c r="K51" s="78" t="n"/>
+      <c r="L51" s="78" t="n"/>
+      <c r="M51" s="74" t="inlineStr">
         <is>
           <t>Скидка возможна только в обмен на ценность: «Готовы дать 5% при оплате счета в течение 24 часов».</t>
         </is>
       </c>
-      <c r="N51" s="73" t="n"/>
-      <c r="O51" s="73" t="n"/>
-      <c r="P51" s="73" t="n"/>
-      <c r="Q51" s="73" t="n"/>
-      <c r="R51" s="73" t="n"/>
-      <c r="S51" s="73" t="n"/>
-      <c r="T51" s="73" t="n"/>
-      <c r="U51" s="73" t="n"/>
-      <c r="V51" s="73" t="n"/>
+      <c r="N51" s="74" t="n"/>
+      <c r="O51" s="74" t="n"/>
+      <c r="P51" s="74" t="n"/>
+      <c r="Q51" s="74" t="n"/>
+      <c r="R51" s="74" t="n"/>
+      <c r="S51" s="74" t="n"/>
+      <c r="T51" s="74" t="n"/>
+      <c r="U51" s="74" t="n"/>
+      <c r="V51" s="74" t="n"/>
     </row>
     <row r="52" ht="12" customHeight="1"/>
     <row r="53" ht="24" customHeight="1">
@@ -4700,215 +4712,215 @@
       <c r="V54" s="25" t="n"/>
     </row>
     <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="79" t="inlineStr">
+      <c r="A55" s="80" t="inlineStr">
         <is>
           <t>Текущие потери от брака звонков в месяц (As-Is)</t>
         </is>
       </c>
-      <c r="B55" s="79" t="n"/>
-      <c r="C55" s="79" t="n"/>
-      <c r="D55" s="80" t="n">
+      <c r="B55" s="80" t="n"/>
+      <c r="C55" s="80" t="n"/>
+      <c r="D55" s="81" t="n">
         <v>1382500</v>
       </c>
-      <c r="E55" s="80" t="n"/>
-      <c r="F55" s="60" t="inlineStr">
+      <c r="E55" s="81" t="n"/>
+      <c r="F55" s="61" t="inlineStr">
         <is>
           <t>Сливы на этапе первичного звонка из-за отсутствия Next Step и слабой отработки возражений</t>
         </is>
       </c>
-      <c r="G55" s="60" t="n"/>
-      <c r="H55" s="60" t="n"/>
-      <c r="I55" s="60" t="n"/>
-      <c r="J55" s="60" t="n"/>
-      <c r="K55" s="60" t="n"/>
-      <c r="L55" s="60" t="n"/>
-      <c r="M55" s="60" t="n"/>
-      <c r="N55" s="60" t="n"/>
-      <c r="O55" s="60" t="n"/>
-      <c r="P55" s="60" t="n"/>
-      <c r="Q55" s="60" t="n"/>
-      <c r="R55" s="60" t="n"/>
-      <c r="S55" s="60" t="n"/>
-      <c r="T55" s="60" t="n"/>
-      <c r="U55" s="60" t="n"/>
-      <c r="V55" s="60" t="n"/>
+      <c r="G55" s="61" t="n"/>
+      <c r="H55" s="61" t="n"/>
+      <c r="I55" s="61" t="n"/>
+      <c r="J55" s="61" t="n"/>
+      <c r="K55" s="61" t="n"/>
+      <c r="L55" s="61" t="n"/>
+      <c r="M55" s="61" t="n"/>
+      <c r="N55" s="61" t="n"/>
+      <c r="O55" s="61" t="n"/>
+      <c r="P55" s="61" t="n"/>
+      <c r="Q55" s="61" t="n"/>
+      <c r="R55" s="61" t="n"/>
+      <c r="S55" s="61" t="n"/>
+      <c r="T55" s="61" t="n"/>
+      <c r="U55" s="61" t="n"/>
+      <c r="V55" s="61" t="n"/>
     </row>
     <row r="56" ht="24" customHeight="1">
-      <c r="A56" s="79" t="inlineStr">
+      <c r="A56" s="80" t="inlineStr">
         <is>
           <t>Ожидаемый возврат выручки в кассу (M1 To-Be)</t>
         </is>
       </c>
-      <c r="B56" s="79" t="n"/>
-      <c r="C56" s="79" t="n"/>
-      <c r="D56" s="81" t="n">
+      <c r="B56" s="80" t="n"/>
+      <c r="C56" s="80" t="n"/>
+      <c r="D56" s="82" t="n">
         <v>414750</v>
       </c>
-      <c r="E56" s="81" t="n"/>
-      <c r="F56" s="60" t="inlineStr">
+      <c r="E56" s="82" t="n"/>
+      <c r="F56" s="61" t="inlineStr">
         <is>
           <t>Консервативный сценарий: устранение всего 30% выявленных дефектов речи</t>
         </is>
       </c>
-      <c r="G56" s="60" t="n"/>
-      <c r="H56" s="60" t="n"/>
-      <c r="I56" s="60" t="n"/>
-      <c r="J56" s="60" t="n"/>
-      <c r="K56" s="60" t="n"/>
-      <c r="L56" s="60" t="n"/>
-      <c r="M56" s="60" t="n"/>
-      <c r="N56" s="60" t="n"/>
-      <c r="O56" s="60" t="n"/>
-      <c r="P56" s="60" t="n"/>
-      <c r="Q56" s="60" t="n"/>
-      <c r="R56" s="60" t="n"/>
-      <c r="S56" s="60" t="n"/>
-      <c r="T56" s="60" t="n"/>
-      <c r="U56" s="60" t="n"/>
-      <c r="V56" s="60" t="n"/>
+      <c r="G56" s="61" t="n"/>
+      <c r="H56" s="61" t="n"/>
+      <c r="I56" s="61" t="n"/>
+      <c r="J56" s="61" t="n"/>
+      <c r="K56" s="61" t="n"/>
+      <c r="L56" s="61" t="n"/>
+      <c r="M56" s="61" t="n"/>
+      <c r="N56" s="61" t="n"/>
+      <c r="O56" s="61" t="n"/>
+      <c r="P56" s="61" t="n"/>
+      <c r="Q56" s="61" t="n"/>
+      <c r="R56" s="61" t="n"/>
+      <c r="S56" s="61" t="n"/>
+      <c r="T56" s="61" t="n"/>
+      <c r="U56" s="61" t="n"/>
+      <c r="V56" s="61" t="n"/>
     </row>
     <row r="57" ht="24" customHeight="1">
-      <c r="A57" s="79" t="inlineStr">
+      <c r="A57" s="80" t="inlineStr">
         <is>
           <t>Стоимость модуля речевого ИИ-супервайзера</t>
         </is>
       </c>
-      <c r="B57" s="79" t="n"/>
-      <c r="C57" s="79" t="n"/>
-      <c r="D57" s="82" t="n">
+      <c r="B57" s="80" t="n"/>
+      <c r="C57" s="80" t="n"/>
+      <c r="D57" s="83" t="n">
         <v>150000</v>
       </c>
-      <c r="E57" s="82" t="n"/>
-      <c r="F57" s="60" t="inlineStr">
+      <c r="E57" s="83" t="n"/>
+      <c r="F57" s="61" t="inlineStr">
         <is>
           <t>В составе комплексного 4-недельного спринта оптимизации отдела продаж</t>
         </is>
       </c>
-      <c r="G57" s="60" t="n"/>
-      <c r="H57" s="60" t="n"/>
-      <c r="I57" s="60" t="n"/>
-      <c r="J57" s="60" t="n"/>
-      <c r="K57" s="60" t="n"/>
-      <c r="L57" s="60" t="n"/>
-      <c r="M57" s="60" t="n"/>
-      <c r="N57" s="60" t="n"/>
-      <c r="O57" s="60" t="n"/>
-      <c r="P57" s="60" t="n"/>
-      <c r="Q57" s="60" t="n"/>
-      <c r="R57" s="60" t="n"/>
-      <c r="S57" s="60" t="n"/>
-      <c r="T57" s="60" t="n"/>
-      <c r="U57" s="60" t="n"/>
-      <c r="V57" s="60" t="n"/>
+      <c r="G57" s="61" t="n"/>
+      <c r="H57" s="61" t="n"/>
+      <c r="I57" s="61" t="n"/>
+      <c r="J57" s="61" t="n"/>
+      <c r="K57" s="61" t="n"/>
+      <c r="L57" s="61" t="n"/>
+      <c r="M57" s="61" t="n"/>
+      <c r="N57" s="61" t="n"/>
+      <c r="O57" s="61" t="n"/>
+      <c r="P57" s="61" t="n"/>
+      <c r="Q57" s="61" t="n"/>
+      <c r="R57" s="61" t="n"/>
+      <c r="S57" s="61" t="n"/>
+      <c r="T57" s="61" t="n"/>
+      <c r="U57" s="61" t="n"/>
+      <c r="V57" s="61" t="n"/>
     </row>
     <row r="58" ht="24" customHeight="1">
-      <c r="A58" s="79" t="inlineStr">
+      <c r="A58" s="80" t="inlineStr">
         <is>
           <t>Чистая прибыль компании от внедрения в первый месяц</t>
         </is>
       </c>
-      <c r="B58" s="79" t="n"/>
-      <c r="C58" s="79" t="n"/>
-      <c r="D58" s="81" t="n">
+      <c r="B58" s="80" t="n"/>
+      <c r="C58" s="80" t="n"/>
+      <c r="D58" s="82" t="n">
         <v>264750</v>
       </c>
-      <c r="E58" s="81" t="n"/>
-      <c r="F58" s="60" t="inlineStr">
+      <c r="E58" s="82" t="n"/>
+      <c r="F58" s="61" t="inlineStr">
         <is>
           <t>Чистый денежный плюс в кассе компании уже в первый месяц работы</t>
         </is>
       </c>
-      <c r="G58" s="60" t="n"/>
-      <c r="H58" s="60" t="n"/>
-      <c r="I58" s="60" t="n"/>
-      <c r="J58" s="60" t="n"/>
-      <c r="K58" s="60" t="n"/>
-      <c r="L58" s="60" t="n"/>
-      <c r="M58" s="60" t="n"/>
-      <c r="N58" s="60" t="n"/>
-      <c r="O58" s="60" t="n"/>
-      <c r="P58" s="60" t="n"/>
-      <c r="Q58" s="60" t="n"/>
-      <c r="R58" s="60" t="n"/>
-      <c r="S58" s="60" t="n"/>
-      <c r="T58" s="60" t="n"/>
-      <c r="U58" s="60" t="n"/>
-      <c r="V58" s="60" t="n"/>
+      <c r="G58" s="61" t="n"/>
+      <c r="H58" s="61" t="n"/>
+      <c r="I58" s="61" t="n"/>
+      <c r="J58" s="61" t="n"/>
+      <c r="K58" s="61" t="n"/>
+      <c r="L58" s="61" t="n"/>
+      <c r="M58" s="61" t="n"/>
+      <c r="N58" s="61" t="n"/>
+      <c r="O58" s="61" t="n"/>
+      <c r="P58" s="61" t="n"/>
+      <c r="Q58" s="61" t="n"/>
+      <c r="R58" s="61" t="n"/>
+      <c r="S58" s="61" t="n"/>
+      <c r="T58" s="61" t="n"/>
+      <c r="U58" s="61" t="n"/>
+      <c r="V58" s="61" t="n"/>
     </row>
     <row r="59" ht="24" customHeight="1">
-      <c r="A59" s="79" t="inlineStr">
+      <c r="A59" s="80" t="inlineStr">
         <is>
           <t>Чистый ROI речевой аналитики</t>
         </is>
       </c>
-      <c r="B59" s="79" t="n"/>
-      <c r="C59" s="79" t="n"/>
-      <c r="D59" s="59" t="inlineStr">
+      <c r="B59" s="80" t="n"/>
+      <c r="C59" s="80" t="n"/>
+      <c r="D59" s="60" t="inlineStr">
         <is>
           <t>276%</t>
         </is>
       </c>
-      <c r="E59" s="59" t="n"/>
-      <c r="F59" s="60" t="inlineStr">
+      <c r="E59" s="60" t="n"/>
+      <c r="F59" s="61" t="inlineStr">
         <is>
           <t>Отдача на каждый вложенный рубль в первый месяц</t>
         </is>
       </c>
-      <c r="G59" s="60" t="n"/>
-      <c r="H59" s="60" t="n"/>
-      <c r="I59" s="60" t="n"/>
-      <c r="J59" s="60" t="n"/>
-      <c r="K59" s="60" t="n"/>
-      <c r="L59" s="60" t="n"/>
-      <c r="M59" s="60" t="n"/>
-      <c r="N59" s="60" t="n"/>
-      <c r="O59" s="60" t="n"/>
-      <c r="P59" s="60" t="n"/>
-      <c r="Q59" s="60" t="n"/>
-      <c r="R59" s="60" t="n"/>
-      <c r="S59" s="60" t="n"/>
-      <c r="T59" s="60" t="n"/>
-      <c r="U59" s="60" t="n"/>
-      <c r="V59" s="60" t="n"/>
+      <c r="G59" s="61" t="n"/>
+      <c r="H59" s="61" t="n"/>
+      <c r="I59" s="61" t="n"/>
+      <c r="J59" s="61" t="n"/>
+      <c r="K59" s="61" t="n"/>
+      <c r="L59" s="61" t="n"/>
+      <c r="M59" s="61" t="n"/>
+      <c r="N59" s="61" t="n"/>
+      <c r="O59" s="61" t="n"/>
+      <c r="P59" s="61" t="n"/>
+      <c r="Q59" s="61" t="n"/>
+      <c r="R59" s="61" t="n"/>
+      <c r="S59" s="61" t="n"/>
+      <c r="T59" s="61" t="n"/>
+      <c r="U59" s="61" t="n"/>
+      <c r="V59" s="61" t="n"/>
     </row>
     <row r="60" ht="24" customHeight="1">
-      <c r="A60" s="79" t="inlineStr">
+      <c r="A60" s="80" t="inlineStr">
         <is>
           <t>Срок полной окупаемости модуля</t>
         </is>
       </c>
-      <c r="B60" s="79" t="n"/>
-      <c r="C60" s="79" t="n"/>
-      <c r="D60" s="59" t="inlineStr">
+      <c r="B60" s="80" t="n"/>
+      <c r="C60" s="80" t="n"/>
+      <c r="D60" s="60" t="inlineStr">
         <is>
           <t>11 дней</t>
         </is>
       </c>
-      <c r="E60" s="59" t="n"/>
-      <c r="F60" s="60" t="inlineStr">
+      <c r="E60" s="60" t="n"/>
+      <c r="F60" s="61" t="inlineStr">
         <is>
           <t>Количество рабочих дней до полной окупаемости внедрения речевого ИИ</t>
         </is>
       </c>
-      <c r="G60" s="60" t="n"/>
-      <c r="H60" s="60" t="n"/>
-      <c r="I60" s="60" t="n"/>
-      <c r="J60" s="60" t="n"/>
-      <c r="K60" s="60" t="n"/>
-      <c r="L60" s="60" t="n"/>
-      <c r="M60" s="60" t="n"/>
-      <c r="N60" s="60" t="n"/>
-      <c r="O60" s="60" t="n"/>
-      <c r="P60" s="60" t="n"/>
-      <c r="Q60" s="60" t="n"/>
-      <c r="R60" s="60" t="n"/>
-      <c r="S60" s="60" t="n"/>
-      <c r="T60" s="60" t="n"/>
-      <c r="U60" s="60" t="n"/>
-      <c r="V60" s="60" t="n"/>
+      <c r="G60" s="61" t="n"/>
+      <c r="H60" s="61" t="n"/>
+      <c r="I60" s="61" t="n"/>
+      <c r="J60" s="61" t="n"/>
+      <c r="K60" s="61" t="n"/>
+      <c r="L60" s="61" t="n"/>
+      <c r="M60" s="61" t="n"/>
+      <c r="N60" s="61" t="n"/>
+      <c r="O60" s="61" t="n"/>
+      <c r="P60" s="61" t="n"/>
+      <c r="Q60" s="61" t="n"/>
+      <c r="R60" s="61" t="n"/>
+      <c r="S60" s="61" t="n"/>
+      <c r="T60" s="61" t="n"/>
+      <c r="U60" s="61" t="n"/>
+      <c r="V60" s="61" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="112">
+  <mergeCells count="113">
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="N2:P2"/>
@@ -4997,6 +5009,7 @@
     <mergeCell ref="M45:V45"/>
     <mergeCell ref="E33:F33"/>
     <mergeCell ref="A56:C56"/>
+    <mergeCell ref="A27:C27"/>
     <mergeCell ref="H50:L50"/>
     <mergeCell ref="F54:V54"/>
     <mergeCell ref="M47:V47"/>
@@ -5046,7 +5059,7 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
@@ -5113,33 +5126,33 @@
           <t>Взвешенный пайплайн в работе</t>
         </is>
       </c>
-      <c r="D4" s="40" t="inlineStr">
+      <c r="D4" s="84" t="inlineStr">
         <is>
           <t>Выявленная упущенная прибыль</t>
         </is>
       </c>
-      <c r="E4" s="83" t="inlineStr">
+      <c r="E4" s="85" t="inlineStr">
         <is>
           <t>Потенциал выручки (To-Be)</t>
         </is>
       </c>
-      <c r="F4" s="83" t="inlineStr">
+      <c r="F4" s="85" t="inlineStr">
         <is>
           <t>Ожидаемый чистый ROI</t>
         </is>
       </c>
-      <c r="G4" s="83" t="inlineStr">
+      <c r="G4" s="85" t="inlineStr">
         <is>
           <t>Срок окупаемости проекта</t>
         </is>
       </c>
-      <c r="H4" s="83" t="n"/>
+      <c r="H4" s="85" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="84" t="n">
+      <c r="A5" s="86" t="n">
         <v>1650000</v>
       </c>
-      <c r="B5" s="84" t="n"/>
+      <c r="B5" s="86" t="n"/>
       <c r="C5" s="23" t="n">
         <v>2754000</v>
       </c>
@@ -5149,17 +5162,17 @@
       <c r="E5" s="22" t="n">
         <v>8651000</v>
       </c>
-      <c r="F5" s="85" t="inlineStr">
+      <c r="F5" s="87" t="inlineStr">
         <is>
           <t>367%</t>
         </is>
       </c>
-      <c r="G5" s="85" t="inlineStr">
+      <c r="G5" s="87" t="inlineStr">
         <is>
           <t>6 дн.</t>
         </is>
       </c>
-      <c r="H5" s="85" t="n"/>
+      <c r="H5" s="87" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -5216,7 +5229,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B9" s="73" t="inlineStr">
+      <c r="B9" s="74" t="inlineStr">
         <is>
           <t>«Черный ящик» CRM: иллюзорный пайплайн</t>
         </is>
@@ -5226,13 +5239,13 @@
           <t>В CRM висит 5.3 млн ₽, но реальный взвешенный объем всего 2.6 млн ₽. Фаундер живет в иллюзии плана</t>
         </is>
       </c>
-      <c r="D9" s="67" t="n">
+      <c r="D9" s="68" t="n">
         <v>5530000</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>2776000</v>
       </c>
-      <c r="F9" s="86" t="inlineStr">
+      <c r="F9" s="88" t="inlineStr">
         <is>
           <t>🔴 P0 (Критический)</t>
         </is>
@@ -5254,7 +5267,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B10" s="73" t="inlineStr">
+      <c r="B10" s="74" t="inlineStr">
         <is>
           <t>«Кладбище сделок»: срыв регламентов SLA</t>
         </is>
@@ -5264,13 +5277,13 @@
           <t>Сделки маринуются на этапе КП по 12–14 дней (норма 48ч). Вероятность закрытия падает на 45%</t>
         </is>
       </c>
-      <c r="D10" s="67" t="n">
+      <c r="D10" s="68" t="n">
         <v>3850000</v>
       </c>
       <c r="E10" s="28" t="n">
         <v>1732500</v>
       </c>
-      <c r="F10" s="86" t="inlineStr">
+      <c r="F10" s="88" t="inlineStr">
         <is>
           <t>🔴 P0 (Критический)</t>
         </is>
@@ -5292,7 +5305,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B11" s="73" t="inlineStr">
+      <c r="B11" s="74" t="inlineStr">
         <is>
           <t>РОП — «играющий тренер» и узкое горлышко</t>
         </is>
@@ -5302,13 +5315,13 @@
           <t>РОП ведет 80% сделок и перегружен (нагрузка 80%), а КАМы простаивают с 4% загрузки. Сделки тухнут без внимания</t>
         </is>
       </c>
-      <c r="D11" s="67" t="n">
+      <c r="D11" s="68" t="n">
         <v>850000</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>255000</v>
       </c>
-      <c r="F11" s="86" t="inlineStr">
+      <c r="F11" s="88" t="inlineStr">
         <is>
           <t>🔴 P0 (Критический)</t>
         </is>
@@ -5330,7 +5343,7 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B12" s="73" t="inlineStr">
+      <c r="B12" s="74" t="inlineStr">
         <is>
           <t>Менеджеры-автоответчики и слив звонков</t>
         </is>
@@ -5340,13 +5353,13 @@
           <t>В 33% звонков не зафиксирован Next Step. Средний балл речи &lt; 9/13. Лиды уходят в «подумаю»</t>
         </is>
       </c>
-      <c r="D12" s="67" t="n">
+      <c r="D12" s="68" t="n">
         <v>5530000</v>
       </c>
       <c r="E12" s="28" t="n">
         <v>1382500</v>
       </c>
-      <c r="F12" s="86" t="inlineStr">
+      <c r="F12" s="88" t="inlineStr">
         <is>
           <t>🔴 P0 (Критический)</t>
         </is>
@@ -5368,7 +5381,7 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B13" s="73" t="inlineStr">
+      <c r="B13" s="74" t="inlineStr">
         <is>
           <t>«Кладбище отказников» без реактивации</t>
         </is>
@@ -5378,13 +5391,13 @@
           <t>1 млн ₽ списан в отказ (L1 «дорого», L2 «подумаю»). База брошена в архиве без повторного прогрева</t>
         </is>
       </c>
-      <c r="D13" s="67" t="n">
+      <c r="D13" s="68" t="n">
         <v>1000000</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>440000</v>
       </c>
-      <c r="F13" s="87" t="inlineStr">
+      <c r="F13" s="89" t="inlineStr">
         <is>
           <t>🟡 P1 (Высокий)</t>
         </is>
@@ -5406,7 +5419,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B14" s="73" t="inlineStr">
+      <c r="B14" s="74" t="inlineStr">
         <is>
           <t>Зависшая дебиторка и кассовые разрывы</t>
         </is>
@@ -5416,13 +5429,13 @@
           <t>Счета выставлены, но не оплачены (DSO &gt; 25 дней). 330к просрочки грозит кассовым разрывом</t>
         </is>
       </c>
-      <c r="D14" s="67" t="n">
+      <c r="D14" s="68" t="n">
         <v>330000</v>
       </c>
       <c r="E14" s="28" t="n">
         <v>330000</v>
       </c>
-      <c r="F14" s="87" t="inlineStr">
+      <c r="F14" s="89" t="inlineStr">
         <is>
           <t>🟡 P1 (Высокий)</t>
         </is>
@@ -5444,7 +5457,7 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B15" s="73" t="inlineStr">
+      <c r="B15" s="74" t="inlineStr">
         <is>
           <t>Слив маркетинга и война с отделом продаж</t>
         </is>
@@ -5454,13 +5467,13 @@
           <t>Google Ads слил 85 000 ₽ с ROMI -100% (0 оплат). Деньги сожжены без сквозного контроля окупаемости</t>
         </is>
       </c>
-      <c r="D15" s="67" t="n">
+      <c r="D15" s="68" t="n">
         <v>850000</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>85000</v>
       </c>
-      <c r="F15" s="87" t="inlineStr">
+      <c r="F15" s="89" t="inlineStr">
         <is>
           <t>🟡 P1 (Высокий)</t>
         </is>
@@ -5484,7 +5497,7 @@
         </is>
       </c>
       <c r="C16" s="29" t="n"/>
-      <c r="D16" s="88">
+      <c r="D16" s="90">
         <f>SUM(D9:D15)</f>
         <v/>
       </c>
@@ -5492,7 +5505,7 @@
         <f>SUM(E9:E15)</f>
         <v/>
       </c>
-      <c r="F16" s="89" t="inlineStr">
+      <c r="F16" s="91" t="inlineStr">
         <is>
           <t>ИТОГО ПОТЕРЬ</t>
         </is>
@@ -5540,7 +5553,7 @@
       </c>
       <c r="B20" s="51" t="n"/>
       <c r="C20" s="51" t="n"/>
-      <c r="D20" s="82" t="n">
+      <c r="D20" s="83" t="n">
         <v>450000</v>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -5560,7 +5573,7 @@
       </c>
       <c r="B21" s="51" t="n"/>
       <c r="C21" s="51" t="n"/>
-      <c r="D21" s="81" t="n">
+      <c r="D21" s="82" t="n">
         <v>2100300</v>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -5580,7 +5593,7 @@
       </c>
       <c r="B22" s="51" t="n"/>
       <c r="C22" s="51" t="n"/>
-      <c r="D22" s="81">
+      <c r="D22" s="82">
         <f>D21-D20</f>
         <v/>
       </c>
@@ -5601,7 +5614,7 @@
       </c>
       <c r="B23" s="51" t="n"/>
       <c r="C23" s="51" t="n"/>
-      <c r="D23" s="59">
+      <c r="D23" s="60">
         <f>(D22/D20)*100 &amp; "%"</f>
         <v/>
       </c>
@@ -5622,7 +5635,7 @@
       </c>
       <c r="B24" s="51" t="n"/>
       <c r="C24" s="51" t="n"/>
-      <c r="D24" s="59">
+      <c r="D24" s="60">
         <f>ROUND(D20/(D21/30), 0) &amp; " дн."</f>
         <v/>
       </c>
@@ -5636,21 +5649,21 @@
       <c r="H24" s="51" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="90" t="inlineStr">
+      <c r="A26" s="92" t="inlineStr">
         <is>
           <t>👉 УТВЕРДИТЬ ПРОЕКТ ОПТИМИЗАЦИИ И СФОРМИРОВАТЬ ИНВОЙС (450 000 ₽)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="91" t="inlineStr">
+      <c r="A27" s="93" t="inlineStr">
         <is>
           <t>Не готовы к спринту? 👉 Бесплатный тест-драйв на 3 звонках на вкладке «⚡ Экспресс_Калькулятор_3_Цифры»</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="92" t="inlineStr">
+      <c r="A28" s="94" t="inlineStr">
         <is>
           <t>🔒 Безопасный B2B-расчет: безналичный платеж по счету (УПД / Диадок) • 152-ФЗ РФ • Старт спринта за 24 часа</t>
         </is>
@@ -5708,7 +5721,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
@@ -5767,24 +5780,24 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="39" t="inlineStr">
+      <c r="A4" s="95" t="inlineStr">
         <is>
           <t>Выручка (Closed-Won)</t>
         </is>
       </c>
-      <c r="B4" s="39" t="inlineStr">
+      <c r="B4" s="95" t="inlineStr">
         <is>
           <t>% Выполнения плана</t>
         </is>
       </c>
-      <c r="C4" s="53" t="inlineStr">
+      <c r="C4" s="96" t="inlineStr">
         <is>
           <t>Взвешенный прогноз</t>
         </is>
       </c>
-      <c r="D4" s="39" t="inlineStr">
-        <is>
-          <t>Run-Rate касса (Прогноз)</t>
+      <c r="D4" s="95" t="inlineStr">
+        <is>
+          <t>Run-Rate касса (мес)</t>
         </is>
       </c>
       <c r="F4" s="39" t="inlineStr">
@@ -5802,14 +5815,14 @@
           <t>Качество речи ОП (ИИ)</t>
         </is>
       </c>
-      <c r="I4" s="83" t="inlineStr">
+      <c r="I4" s="85" t="inlineStr">
         <is>
           <t>Data Quality Index</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="84" t="n">
+      <c r="A5" s="86" t="n">
         <v>1650000</v>
       </c>
       <c r="B5" s="41" t="inlineStr">
@@ -5820,10 +5833,10 @@
       <c r="C5" s="23" t="n">
         <v>2754000</v>
       </c>
-      <c r="D5" s="84" t="n">
+      <c r="D5" s="86" t="n">
         <v>1706897</v>
       </c>
-      <c r="F5" s="84" t="n">
+      <c r="F5" s="86" t="n">
         <v>5530000</v>
       </c>
       <c r="G5" s="42" t="inlineStr">
@@ -5836,7 +5849,7 @@
           <t>73.1%</t>
         </is>
       </c>
-      <c r="I5" s="85" t="inlineStr">
+      <c r="I5" s="87" t="inlineStr">
         <is>
           <t>100.0% (Эталон)</t>
         </is>
@@ -5911,7 +5924,7 @@
       <c r="D9" s="26" t="n">
         <v>24</v>
       </c>
-      <c r="F9" s="79" t="inlineStr">
+      <c r="F9" s="80" t="inlineStr">
         <is>
           <t>D-104 (ООО Вектор)</t>
         </is>
@@ -5921,7 +5934,7 @@
           <t>КП без ответа &gt; 48ч</t>
         </is>
       </c>
-      <c r="H9" s="61" t="n">
+      <c r="H9" s="62" t="n">
         <v>850000</v>
       </c>
       <c r="I9" s="27" t="inlineStr">
@@ -5945,7 +5958,7 @@
       <c r="D10" s="26" t="n">
         <v>48</v>
       </c>
-      <c r="F10" s="79" t="inlineStr">
+      <c r="F10" s="80" t="inlineStr">
         <is>
           <t>D-103 (ИнвестХолдинг)</t>
         </is>
@@ -5955,7 +5968,7 @@
           <t>Просрочен счёт на оплату</t>
         </is>
       </c>
-      <c r="H10" s="61" t="n">
+      <c r="H10" s="62" t="n">
         <v>150000</v>
       </c>
       <c r="I10" s="27" t="inlineStr">
@@ -5979,7 +5992,7 @@
       <c r="D11" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="F11" s="79" t="inlineStr">
+      <c r="F11" s="80" t="inlineStr">
         <is>
           <t>D-109 (ПромКомплект)</t>
         </is>
@@ -5989,7 +6002,7 @@
           <t>Критический брак речи (&lt;9)</t>
         </is>
       </c>
-      <c r="H11" s="61" t="n">
+      <c r="H11" s="62" t="n">
         <v>600000</v>
       </c>
       <c r="I11" s="27" t="inlineStr">
@@ -6013,7 +6026,7 @@
       <c r="D12" s="26" t="n">
         <v>48</v>
       </c>
-      <c r="F12" s="79" t="inlineStr">
+      <c r="F12" s="80" t="inlineStr">
         <is>
           <t>D-106 (СнабСервис)</t>
         </is>
@@ -6023,7 +6036,7 @@
           <t>Зависание на этапе КП</t>
         </is>
       </c>
-      <c r="H12" s="61" t="n">
+      <c r="H12" s="62" t="n">
         <v>280000</v>
       </c>
       <c r="I12" s="27" t="inlineStr">
@@ -6047,7 +6060,7 @@
       <c r="D13" s="26" t="n">
         <v>72</v>
       </c>
-      <c r="F13" s="79" t="inlineStr">
+      <c r="F13" s="80" t="inlineStr">
         <is>
           <t>D-107 (ТехноПром)</t>
         </is>
@@ -6057,7 +6070,7 @@
           <t>Крупная сделка без движения</t>
         </is>
       </c>
-      <c r="H13" s="61" t="n">
+      <c r="H13" s="62" t="n">
         <v>3000000</v>
       </c>
       <c r="I13" s="27" t="inlineStr">
@@ -6083,19 +6096,19 @@
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="93" t="inlineStr">
+      <c r="A16" s="97" t="inlineStr">
         <is>
           <t>🎯 ГЛАВНЫЙ ФОКУС РУКОВОДСТВА ДО КОНЦА МЕСЯЦА: Перехват сделки D-104 (850 000 ₽) и перераспределение 3 лидов с перегруженного РОПа на КАМов.</t>
         </is>
       </c>
-      <c r="B16" s="93" t="n"/>
-      <c r="C16" s="93" t="n"/>
-      <c r="D16" s="93" t="n"/>
-      <c r="E16" s="93" t="n"/>
-      <c r="F16" s="93" t="n"/>
-      <c r="G16" s="93" t="n"/>
-      <c r="H16" s="93" t="n"/>
-      <c r="I16" s="93" t="n"/>
+      <c r="B16" s="97" t="n"/>
+      <c r="C16" s="97" t="n"/>
+      <c r="D16" s="97" t="n"/>
+      <c r="E16" s="97" t="n"/>
+      <c r="F16" s="97" t="n"/>
+      <c r="G16" s="97" t="n"/>
+      <c r="H16" s="97" t="n"/>
+      <c r="I16" s="97" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -6151,32 +6164,32 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>⚡ Экспресс-Калькулятор</t>
+          <t>⚡ Калькулятор</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>📋 Пульт РОПа (15 мин)</t>
+          <t>📋 Пульт РОПа</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>🎙️ ИИ-Аудит звонков</t>
+          <t>🎙️ ИИ-Аудит</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>💸 7 Грехов (Диагностика)</t>
+          <t>💸 7 Грехов ОП</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>📄 Executive One-Pager</t>
+          <t>📄 One-Pager</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>🔐 152-ФЗ Безопасность</t>
+          <t>🔐 152-ФЗ</t>
         </is>
       </c>
     </row>
@@ -6223,7 +6236,7 @@
       <c r="A6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="73" t="inlineStr">
+      <c r="B6" s="74" t="inlineStr">
         <is>
           <t>Локализация баз данных</t>
         </is>
@@ -6238,7 +6251,7 @@
           <t>Дата-центры в Москве (Yandex Cloud / Selectel), аттестация ФСТЭК УЗ 1-2</t>
         </is>
       </c>
-      <c r="E6" s="85" t="inlineStr">
+      <c r="E6" s="87" t="inlineStr">
         <is>
           <t>✅ 100% Соответствие</t>
         </is>
@@ -6253,7 +6266,7 @@
       <c r="A7" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="73" t="inlineStr">
+      <c r="B7" s="74" t="inlineStr">
         <is>
           <t>Криптографическая токенизация</t>
         </is>
@@ -6268,7 +6281,7 @@
           <t>Модуль PIISanitizer: замена телефонов, ФИО и карт на токены [PHONE_TOKEN_X]</t>
         </is>
       </c>
-      <c r="E7" s="85" t="inlineStr">
+      <c r="E7" s="87" t="inlineStr">
         <is>
           <t>✅ Автоматически</t>
         </is>
@@ -6283,7 +6296,7 @@
       <c r="A8" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="73" t="inlineStr">
+      <c r="B8" s="74" t="inlineStr">
         <is>
           <t>Срок хранения аудиозаписей</t>
         </is>
@@ -6298,7 +6311,7 @@
           <t>Автоматическое безвозвратное удаление исходных аудио через 30 дней</t>
         </is>
       </c>
-      <c r="E8" s="85" t="inlineStr">
+      <c r="E8" s="87" t="inlineStr">
         <is>
           <t>✅ Настроено в cron</t>
         </is>
@@ -6313,7 +6326,7 @@
       <c r="A9" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="73" t="inlineStr">
+      <c r="B9" s="74" t="inlineStr">
         <is>
           <t>Согласие сотрудников ОП</t>
         </is>
@@ -6328,7 +6341,7 @@
           <t>Готовый пакет документов: Приказ, Положение о контроле, Согласие</t>
         </is>
       </c>
-      <c r="E9" s="85" t="inlineStr">
+      <c r="E9" s="87" t="inlineStr">
         <is>
           <t>✅ Комплект включен</t>
         </is>
@@ -6343,7 +6356,7 @@
       <c r="A10" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="73" t="inlineStr">
+      <c r="B10" s="74" t="inlineStr">
         <is>
           <t>Юридический статус исполнителя</t>
         </is>
@@ -6358,7 +6371,7 @@
           <t>Плательщик НПД (Самозанятый), чек приложения «Мой Налог», договор, акт</t>
         </is>
       </c>
-      <c r="E10" s="85" t="inlineStr">
+      <c r="E10" s="87" t="inlineStr">
         <is>
           <t>✅ Безопасно для бухгалтерии</t>
         </is>
@@ -6373,7 +6386,7 @@
       <c r="A11" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="73" t="inlineStr">
+      <c r="B11" s="74" t="inlineStr">
         <is>
           <t>Гарантия конфиденциальности NDA</t>
         </is>
@@ -6388,7 +6401,7 @@
           <t>Подписание двустороннего соглашения о неразглашении конфиденциальных данных</t>
         </is>
       </c>
-      <c r="E11" s="85" t="inlineStr">
+      <c r="E11" s="87" t="inlineStr">
         <is>
           <t>✅ Подписание в ЭДО</t>
         </is>

</xml_diff>

<commit_message>
style: capital polish of Google Sheets and Excel presentation workbook (row heights, borders, aligned anchors, dynamic formulas)
</commit_message>
<xml_diff>
--- a/docs/RevOps_Platform_Demo_Sample.xlsx
+++ b/docs/RevOps_Platform_Demo_Sample.xlsx
@@ -1207,8 +1207,9 @@
           <t>30% выручки теряется из-за ошибок менеджеров</t>
         </is>
       </c>
-      <c r="D15" s="28" t="n">
-        <v>412500</v>
+      <c r="D15" s="28">
+        <f>ROUND(H6*0.3968, -2)</f>
+        <v/>
       </c>
       <c r="E15" s="27" t="inlineStr">
         <is>
@@ -1237,8 +1238,9 @@
           <t>18% выручки теряется из-за просрочки follow-up</t>
         </is>
       </c>
-      <c r="D16" s="28" t="n">
-        <v>297000</v>
+      <c r="D16" s="28">
+        <f>ROUND(H6*0.2857, -2)</f>
+        <v/>
       </c>
       <c r="E16" s="27" t="inlineStr">
         <is>
@@ -1267,8 +1269,9 @@
           <t>8% — потенциал реактивации списанных сделок</t>
         </is>
       </c>
-      <c r="D17" s="28" t="n">
-        <v>132000</v>
+      <c r="D17" s="28">
+        <f>ROUND(H6*0.1270, -2)</f>
+        <v/>
       </c>
       <c r="E17" s="27" t="inlineStr">
         <is>
@@ -1297,8 +1300,9 @@
           <t>12% выставленных счетов с просрочкой 20+ дней</t>
         </is>
       </c>
-      <c r="D18" s="28" t="n">
-        <v>198000</v>
+      <c r="D18" s="28">
+        <f>H6-D15-D16-D17</f>
+        <v/>
       </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
@@ -3665,7 +3669,7 @@
       <c r="U30" s="25" t="n"/>
       <c r="V30" s="25" t="n"/>
     </row>
-    <row r="31" ht="54" customHeight="1">
+    <row r="31" ht="60" customHeight="1">
       <c r="A31" s="44" t="inlineStr">
         <is>
           <t>C-505</t>
@@ -3715,7 +3719,7 @@
       <c r="U31" s="77" t="n"/>
       <c r="V31" s="77" t="n"/>
     </row>
-    <row r="32" ht="54" customHeight="1">
+    <row r="32" ht="60" customHeight="1">
       <c r="A32" s="44" t="inlineStr">
         <is>
           <t>C-503</t>
@@ -3765,7 +3769,7 @@
       <c r="U32" s="77" t="n"/>
       <c r="V32" s="77" t="n"/>
     </row>
-    <row r="33" ht="54" customHeight="1">
+    <row r="33" ht="60" customHeight="1">
       <c r="A33" s="44" t="inlineStr">
         <is>
           <t>C-507</t>
@@ -3815,7 +3819,7 @@
       <c r="U33" s="77" t="n"/>
       <c r="V33" s="77" t="n"/>
     </row>
-    <row r="34" ht="54" customHeight="1">
+    <row r="34" ht="60" customHeight="1">
       <c r="A34" s="44" t="inlineStr">
         <is>
           <t>C-508</t>
@@ -3865,7 +3869,7 @@
       <c r="U34" s="77" t="n"/>
       <c r="V34" s="77" t="n"/>
     </row>
-    <row r="35" ht="54" customHeight="1">
+    <row r="35" ht="60" customHeight="1">
       <c r="A35" s="44" t="inlineStr">
         <is>
           <t>C-510</t>
@@ -3996,7 +4000,7 @@
       <c r="U38" s="25" t="n"/>
       <c r="V38" s="25" t="n"/>
     </row>
-    <row r="39" ht="34" customHeight="1">
+    <row r="39" ht="46" customHeight="1">
       <c r="A39" s="26" t="n">
         <v>1</v>
       </c>
@@ -4046,7 +4050,7 @@
       <c r="U39" s="74" t="n"/>
       <c r="V39" s="74" t="n"/>
     </row>
-    <row r="40" ht="34" customHeight="1">
+    <row r="40" ht="46" customHeight="1">
       <c r="A40" s="26" t="n">
         <v>2</v>
       </c>
@@ -4096,7 +4100,7 @@
       <c r="U40" s="74" t="n"/>
       <c r="V40" s="74" t="n"/>
     </row>
-    <row r="41" ht="34" customHeight="1">
+    <row r="41" ht="46" customHeight="1">
       <c r="A41" s="26" t="n">
         <v>3</v>
       </c>
@@ -4146,7 +4150,7 @@
       <c r="U41" s="74" t="n"/>
       <c r="V41" s="74" t="n"/>
     </row>
-    <row r="42" ht="34" customHeight="1">
+    <row r="42" ht="46" customHeight="1">
       <c r="A42" s="26" t="n">
         <v>4</v>
       </c>
@@ -4196,7 +4200,7 @@
       <c r="U42" s="74" t="n"/>
       <c r="V42" s="74" t="n"/>
     </row>
-    <row r="43" ht="34" customHeight="1">
+    <row r="43" ht="46" customHeight="1">
       <c r="A43" s="26" t="n">
         <v>5</v>
       </c>
@@ -4246,7 +4250,7 @@
       <c r="U43" s="74" t="n"/>
       <c r="V43" s="74" t="n"/>
     </row>
-    <row r="44" ht="34" customHeight="1">
+    <row r="44" ht="46" customHeight="1">
       <c r="A44" s="26" t="n">
         <v>6</v>
       </c>
@@ -4296,7 +4300,7 @@
       <c r="U44" s="74" t="n"/>
       <c r="V44" s="74" t="n"/>
     </row>
-    <row r="45" ht="34" customHeight="1">
+    <row r="45" ht="46" customHeight="1">
       <c r="A45" s="26" t="n">
         <v>7</v>
       </c>
@@ -4346,7 +4350,7 @@
       <c r="U45" s="74" t="n"/>
       <c r="V45" s="74" t="n"/>
     </row>
-    <row r="46" ht="34" customHeight="1">
+    <row r="46" ht="46" customHeight="1">
       <c r="A46" s="26" t="n">
         <v>8</v>
       </c>
@@ -4396,7 +4400,7 @@
       <c r="U46" s="74" t="n"/>
       <c r="V46" s="74" t="n"/>
     </row>
-    <row r="47" ht="34" customHeight="1">
+    <row r="47" ht="46" customHeight="1">
       <c r="A47" s="26" t="n">
         <v>9</v>
       </c>
@@ -4446,7 +4450,7 @@
       <c r="U47" s="74" t="n"/>
       <c r="V47" s="74" t="n"/>
     </row>
-    <row r="48" ht="34" customHeight="1">
+    <row r="48" ht="46" customHeight="1">
       <c r="A48" s="26" t="n">
         <v>10</v>
       </c>
@@ -4496,7 +4500,7 @@
       <c r="U48" s="74" t="n"/>
       <c r="V48" s="74" t="n"/>
     </row>
-    <row r="49" ht="34" customHeight="1">
+    <row r="49" ht="46" customHeight="1">
       <c r="A49" s="26" t="n">
         <v>11</v>
       </c>
@@ -4546,7 +4550,7 @@
       <c r="U49" s="74" t="n"/>
       <c r="V49" s="74" t="n"/>
     </row>
-    <row r="50" ht="34" customHeight="1">
+    <row r="50" ht="46" customHeight="1">
       <c r="A50" s="26" t="n">
         <v>12</v>
       </c>
@@ -4596,7 +4600,7 @@
       <c r="U50" s="74" t="n"/>
       <c r="V50" s="74" t="n"/>
     </row>
-    <row r="51" ht="34" customHeight="1">
+    <row r="51" ht="46" customHeight="1">
       <c r="A51" s="26" t="n">
         <v>13</v>
       </c>

</xml_diff>